<commit_message>
feat: add map parser and showcase coverage
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Core.xlsx
+++ b/examples/showcase/data/Core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="1032">
   <si>
     <t>@table</t>
   </si>
@@ -2723,6 +2723,396 @@
   </si>
   <si>
     <t>feature_100</t>
+  </si>
+  <si>
+    <t>6032309d1d0279cc</t>
+  </si>
+  <si>
+    <t>attributes</t>
+  </si>
+  <si>
+    <t>set&lt;string&gt;</t>
+  </si>
+  <si>
+    <t>map&lt;string,i32&gt;</t>
+  </si>
+  <si>
+    <t>optional;parser=json</t>
+  </si>
+  <si>
+    <t>required;parser=map</t>
+  </si>
+  <si>
+    <t>JSON string set</t>
+  </si>
+  <si>
+    <t>Map pairs: key,value|key,value</t>
+  </si>
+  <si>
+    <t>tier,1|power,10</t>
+  </si>
+  <si>
+    <t>tier,2|power,11</t>
+  </si>
+  <si>
+    <t>tier,3|power,12</t>
+  </si>
+  <si>
+    <t>tier,4|power,13</t>
+  </si>
+  <si>
+    <t>tier,5|power,14</t>
+  </si>
+  <si>
+    <t>tier,1|power,15</t>
+  </si>
+  <si>
+    <t>tier,2|power,16</t>
+  </si>
+  <si>
+    <t>tier,3|power,17</t>
+  </si>
+  <si>
+    <t>tier,4|power,18</t>
+  </si>
+  <si>
+    <t>tier,5|power,19</t>
+  </si>
+  <si>
+    <t>tier,1|power,20</t>
+  </si>
+  <si>
+    <t>tier,2|power,21</t>
+  </si>
+  <si>
+    <t>tier,3|power,22</t>
+  </si>
+  <si>
+    <t>tier,4|power,23</t>
+  </si>
+  <si>
+    <t>tier,5|power,24</t>
+  </si>
+  <si>
+    <t>tier,1|power,25</t>
+  </si>
+  <si>
+    <t>tier,2|power,26</t>
+  </si>
+  <si>
+    <t>tier,3|power,27</t>
+  </si>
+  <si>
+    <t>tier,4|power,28</t>
+  </si>
+  <si>
+    <t>tier,5|power,29</t>
+  </si>
+  <si>
+    <t>tier,1|power,30</t>
+  </si>
+  <si>
+    <t>tier,2|power,31</t>
+  </si>
+  <si>
+    <t>tier,3|power,32</t>
+  </si>
+  <si>
+    <t>tier,4|power,33</t>
+  </si>
+  <si>
+    <t>tier,5|power,34</t>
+  </si>
+  <si>
+    <t>tier,1|power,35</t>
+  </si>
+  <si>
+    <t>tier,2|power,36</t>
+  </si>
+  <si>
+    <t>tier,3|power,37</t>
+  </si>
+  <si>
+    <t>tier,4|power,38</t>
+  </si>
+  <si>
+    <t>tier,5|power,39</t>
+  </si>
+  <si>
+    <t>tier,1|power,40</t>
+  </si>
+  <si>
+    <t>tier,2|power,41</t>
+  </si>
+  <si>
+    <t>tier,3|power,42</t>
+  </si>
+  <si>
+    <t>tier,4|power,43</t>
+  </si>
+  <si>
+    <t>tier,5|power,44</t>
+  </si>
+  <si>
+    <t>tier,1|power,45</t>
+  </si>
+  <si>
+    <t>tier,2|power,46</t>
+  </si>
+  <si>
+    <t>tier,3|power,47</t>
+  </si>
+  <si>
+    <t>tier,4|power,48</t>
+  </si>
+  <si>
+    <t>tier,5|power,49</t>
+  </si>
+  <si>
+    <t>tier,1|power,50</t>
+  </si>
+  <si>
+    <t>tier,2|power,51</t>
+  </si>
+  <si>
+    <t>tier,3|power,52</t>
+  </si>
+  <si>
+    <t>tier,4|power,53</t>
+  </si>
+  <si>
+    <t>tier,5|power,54</t>
+  </si>
+  <si>
+    <t>tier,1|power,55</t>
+  </si>
+  <si>
+    <t>tier,2|power,56</t>
+  </si>
+  <si>
+    <t>tier,3|power,57</t>
+  </si>
+  <si>
+    <t>tier,4|power,58</t>
+  </si>
+  <si>
+    <t>tier,5|power,59</t>
+  </si>
+  <si>
+    <t>tier,1|power,60</t>
+  </si>
+  <si>
+    <t>tier,2|power,61</t>
+  </si>
+  <si>
+    <t>tier,3|power,62</t>
+  </si>
+  <si>
+    <t>tier,4|power,63</t>
+  </si>
+  <si>
+    <t>tier,5|power,64</t>
+  </si>
+  <si>
+    <t>tier,1|power,65</t>
+  </si>
+  <si>
+    <t>tier,2|power,66</t>
+  </si>
+  <si>
+    <t>tier,3|power,67</t>
+  </si>
+  <si>
+    <t>tier,4|power,68</t>
+  </si>
+  <si>
+    <t>tier,5|power,69</t>
+  </si>
+  <si>
+    <t>tier,1|power,70</t>
+  </si>
+  <si>
+    <t>tier,2|power,71</t>
+  </si>
+  <si>
+    <t>tier,3|power,72</t>
+  </si>
+  <si>
+    <t>tier,4|power,73</t>
+  </si>
+  <si>
+    <t>tier,5|power,74</t>
+  </si>
+  <si>
+    <t>tier,1|power,75</t>
+  </si>
+  <si>
+    <t>tier,2|power,76</t>
+  </si>
+  <si>
+    <t>tier,3|power,77</t>
+  </si>
+  <si>
+    <t>tier,4|power,78</t>
+  </si>
+  <si>
+    <t>tier,5|power,79</t>
+  </si>
+  <si>
+    <t>tier,1|power,80</t>
+  </si>
+  <si>
+    <t>tier,2|power,81</t>
+  </si>
+  <si>
+    <t>tier,3|power,82</t>
+  </si>
+  <si>
+    <t>tier,4|power,83</t>
+  </si>
+  <si>
+    <t>tier,5|power,84</t>
+  </si>
+  <si>
+    <t>tier,1|power,85</t>
+  </si>
+  <si>
+    <t>tier,2|power,86</t>
+  </si>
+  <si>
+    <t>tier,3|power,87</t>
+  </si>
+  <si>
+    <t>tier,4|power,88</t>
+  </si>
+  <si>
+    <t>tier,5|power,89</t>
+  </si>
+  <si>
+    <t>tier,1|power,90</t>
+  </si>
+  <si>
+    <t>tier,2|power,91</t>
+  </si>
+  <si>
+    <t>tier,3|power,92</t>
+  </si>
+  <si>
+    <t>tier,4|power,93</t>
+  </si>
+  <si>
+    <t>tier,5|power,94</t>
+  </si>
+  <si>
+    <t>tier,1|power,95</t>
+  </si>
+  <si>
+    <t>tier,2|power,96</t>
+  </si>
+  <si>
+    <t>tier,3|power,97</t>
+  </si>
+  <si>
+    <t>tier,4|power,98</t>
+  </si>
+  <si>
+    <t>tier,5|power,99</t>
+  </si>
+  <si>
+    <t>tier,1|power,100</t>
+  </si>
+  <si>
+    <t>tier,2|power,101</t>
+  </si>
+  <si>
+    <t>tier,3|power,102</t>
+  </si>
+  <si>
+    <t>tier,4|power,103</t>
+  </si>
+  <si>
+    <t>tier,5|power,104</t>
+  </si>
+  <si>
+    <t>tier,1|power,105</t>
+  </si>
+  <si>
+    <t>tier,2|power,106</t>
+  </si>
+  <si>
+    <t>tier,3|power,107</t>
+  </si>
+  <si>
+    <t>tier,4|power,108</t>
+  </si>
+  <si>
+    <t>tier,5|power,109</t>
+  </si>
+  <si>
+    <t>tier,1|power,110</t>
+  </si>
+  <si>
+    <t>tier,2|power,111</t>
+  </si>
+  <si>
+    <t>tier,3|power,112</t>
+  </si>
+  <si>
+    <t>tier,4|power,113</t>
+  </si>
+  <si>
+    <t>tier,5|power,114</t>
+  </si>
+  <si>
+    <t>tier,1|power,115</t>
+  </si>
+  <si>
+    <t>tier,2|power,116</t>
+  </si>
+  <si>
+    <t>tier,3|power,117</t>
+  </si>
+  <si>
+    <t>tier,4|power,118</t>
+  </si>
+  <si>
+    <t>tier,5|power,119</t>
+  </si>
+  <si>
+    <t>tier,1|power,120</t>
+  </si>
+  <si>
+    <t>tier,2|power,121</t>
+  </si>
+  <si>
+    <t>tier,3|power,122</t>
+  </si>
+  <si>
+    <t>tier,4|power,123</t>
+  </si>
+  <si>
+    <t>tier,5|power,124</t>
+  </si>
+  <si>
+    <t>tier,1|power,125</t>
+  </si>
+  <si>
+    <t>tier,2|power,126</t>
+  </si>
+  <si>
+    <t>tier,3|power,127</t>
+  </si>
+  <si>
+    <t>tier,4|power,128</t>
+  </si>
+  <si>
+    <t>tier,5|power,129</t>
+  </si>
+  <si>
+    <t>tier,1|power,130</t>
+  </si>
+  <si>
+    <t>tier,2|power,131</t>
   </si>
 </sst>
 </file>
@@ -3053,8 +3443,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G134"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3089,15 +3479,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3119,8 +3509,11 @@
       <c r="G7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3142,8 +3535,11 @@
       <c r="G8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="H8" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -3163,10 +3559,13 @@
         <v>21</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>904</v>
+      </c>
+      <c r="H9" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -3188,8 +3587,11 @@
       <c r="G10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -3209,10 +3611,13 @@
         <v>28</v>
       </c>
       <c r="G11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>906</v>
+      </c>
+      <c r="H11" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -3232,7 +3637,10 @@
         <v>35</v>
       </c>
       <c r="G12" t="s">
-        <v>36</v>
+        <v>908</v>
+      </c>
+      <c r="H12" t="s">
+        <v>909</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -3254,6 +3662,9 @@
       <c r="F13" t="s">
         <v>42</v>
       </c>
+      <c r="G13" t="s">
+        <v>910</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
@@ -3274,6 +3685,9 @@
       <c r="F14" t="s">
         <v>48</v>
       </c>
+      <c r="G14" t="s">
+        <v>911</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
@@ -3294,6 +3708,9 @@
       <c r="F15" t="s">
         <v>54</v>
       </c>
+      <c r="G15" t="s">
+        <v>912</v>
+      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
@@ -3311,8 +3728,11 @@
       <c r="F16" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>60</v>
       </c>
@@ -3331,8 +3751,11 @@
       <c r="F17" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>65</v>
       </c>
@@ -3351,8 +3774,11 @@
       <c r="F18" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="G18" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -3371,8 +3797,11 @@
       <c r="F19" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -3391,8 +3820,11 @@
       <c r="F20" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>79</v>
       </c>
@@ -3411,8 +3843,11 @@
       <c r="F21" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>84</v>
       </c>
@@ -3431,8 +3866,11 @@
       <c r="F22" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>88</v>
       </c>
@@ -3451,8 +3889,11 @@
       <c r="F23" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="G23" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>92</v>
       </c>
@@ -3471,8 +3912,11 @@
       <c r="F24" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>95</v>
       </c>
@@ -3491,8 +3935,11 @@
       <c r="F25" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="G25" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>98</v>
       </c>
@@ -3511,8 +3958,11 @@
       <c r="F26" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="G26" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>102</v>
       </c>
@@ -3531,8 +3981,11 @@
       <c r="F27" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="G27" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>106</v>
       </c>
@@ -3551,8 +4004,11 @@
       <c r="F28" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="G28" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>110</v>
       </c>
@@ -3571,8 +4027,11 @@
       <c r="F29" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="G29" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>112</v>
       </c>
@@ -3591,8 +4050,11 @@
       <c r="F30" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="G30" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>115</v>
       </c>
@@ -3611,8 +4073,11 @@
       <c r="F31" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="G31" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>119</v>
       </c>
@@ -3631,8 +4096,11 @@
       <c r="F32" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="G32" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>123</v>
       </c>
@@ -3651,8 +4119,11 @@
       <c r="F33" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="G33" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>127</v>
       </c>
@@ -3671,8 +4142,11 @@
       <c r="F34" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="G34" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>130</v>
       </c>
@@ -3691,8 +4165,11 @@
       <c r="F35" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>133</v>
       </c>
@@ -3711,8 +4188,11 @@
       <c r="F36" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="G36" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>137</v>
       </c>
@@ -3731,8 +4211,11 @@
       <c r="F37" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="G37" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>141</v>
       </c>
@@ -3751,8 +4234,11 @@
       <c r="F38" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>145</v>
       </c>
@@ -3771,8 +4257,11 @@
       <c r="F39" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39" t="s">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>148</v>
       </c>
@@ -3791,8 +4280,11 @@
       <c r="F40" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="G40" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>151</v>
       </c>
@@ -3811,8 +4303,11 @@
       <c r="F41" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="G41" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>155</v>
       </c>
@@ -3831,8 +4326,11 @@
       <c r="F42" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
+      <c r="G42" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>159</v>
       </c>
@@ -3851,8 +4349,11 @@
       <c r="F43" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="44" spans="1:6">
+      <c r="G43" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>163</v>
       </c>
@@ -3871,8 +4372,11 @@
       <c r="F44" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="45" spans="1:6">
+      <c r="G44" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>166</v>
       </c>
@@ -3891,8 +4395,11 @@
       <c r="F45" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="46" spans="1:6">
+      <c r="G45" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>169</v>
       </c>
@@ -3911,8 +4418,11 @@
       <c r="F46" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="47" spans="1:6">
+      <c r="G46" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>173</v>
       </c>
@@ -3931,8 +4441,11 @@
       <c r="F47" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="48" spans="1:6">
+      <c r="G47" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>177</v>
       </c>
@@ -3951,8 +4464,11 @@
       <c r="F48" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="49" spans="1:6">
+      <c r="G48" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
         <v>181</v>
       </c>
@@ -3971,8 +4487,11 @@
       <c r="F49" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="50" spans="1:6">
+      <c r="G49" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>184</v>
       </c>
@@ -3991,8 +4510,11 @@
       <c r="F50" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="51" spans="1:6">
+      <c r="G50" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>187</v>
       </c>
@@ -4011,8 +4533,11 @@
       <c r="F51" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="52" spans="1:6">
+      <c r="G51" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>191</v>
       </c>
@@ -4031,8 +4556,11 @@
       <c r="F52" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="53" spans="1:6">
+      <c r="G52" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
         <v>195</v>
       </c>
@@ -4051,8 +4579,11 @@
       <c r="F53" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="54" spans="1:6">
+      <c r="G53" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>198</v>
       </c>
@@ -4071,8 +4602,11 @@
       <c r="F54" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="55" spans="1:6">
+      <c r="G54" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
         <v>201</v>
       </c>
@@ -4091,8 +4625,11 @@
       <c r="F55" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="56" spans="1:6">
+      <c r="G55" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>204</v>
       </c>
@@ -4111,8 +4648,11 @@
       <c r="F56" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="57" spans="1:6">
+      <c r="G56" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>208</v>
       </c>
@@ -4131,8 +4671,11 @@
       <c r="F57" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="58" spans="1:6">
+      <c r="G57" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>212</v>
       </c>
@@ -4151,8 +4694,11 @@
       <c r="F58" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="59" spans="1:6">
+      <c r="G58" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>216</v>
       </c>
@@ -4171,8 +4717,11 @@
       <c r="F59" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="60" spans="1:6">
+      <c r="G59" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>219</v>
       </c>
@@ -4191,8 +4740,11 @@
       <c r="F60" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="61" spans="1:6">
+      <c r="G60" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
         <v>222</v>
       </c>
@@ -4211,8 +4763,11 @@
       <c r="F61" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="62" spans="1:6">
+      <c r="G61" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
         <v>226</v>
       </c>
@@ -4231,8 +4786,11 @@
       <c r="F62" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="63" spans="1:6">
+      <c r="G62" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
         <v>230</v>
       </c>
@@ -4251,8 +4809,11 @@
       <c r="F63" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="64" spans="1:6">
+      <c r="G63" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
         <v>234</v>
       </c>
@@ -4271,8 +4832,11 @@
       <c r="F64" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="65" spans="1:6">
+      <c r="G64" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
       <c r="A65" t="s">
         <v>237</v>
       </c>
@@ -4291,8 +4855,11 @@
       <c r="F65" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="G65" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
       <c r="A66" t="s">
         <v>240</v>
       </c>
@@ -4311,8 +4878,11 @@
       <c r="F66" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="67" spans="1:6">
+      <c r="G66" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
       <c r="A67" t="s">
         <v>244</v>
       </c>
@@ -4331,8 +4901,11 @@
       <c r="F67" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="68" spans="1:6">
+      <c r="G67" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
       <c r="A68" t="s">
         <v>248</v>
       </c>
@@ -4351,8 +4924,11 @@
       <c r="F68" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="69" spans="1:6">
+      <c r="G68" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
       <c r="A69" t="s">
         <v>252</v>
       </c>
@@ -4371,8 +4947,11 @@
       <c r="F69" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="70" spans="1:6">
+      <c r="G69" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
       <c r="A70" t="s">
         <v>255</v>
       </c>
@@ -4391,8 +4970,11 @@
       <c r="F70" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="71" spans="1:6">
+      <c r="G70" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
       <c r="A71" t="s">
         <v>258</v>
       </c>
@@ -4411,8 +4993,11 @@
       <c r="F71" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="72" spans="1:6">
+      <c r="G71" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7">
       <c r="A72" t="s">
         <v>262</v>
       </c>
@@ -4431,8 +5016,11 @@
       <c r="F72" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="73" spans="1:6">
+      <c r="G72" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7">
       <c r="A73" t="s">
         <v>266</v>
       </c>
@@ -4451,8 +5039,11 @@
       <c r="F73" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="74" spans="1:6">
+      <c r="G73" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7">
       <c r="A74" t="s">
         <v>270</v>
       </c>
@@ -4471,8 +5062,11 @@
       <c r="F74" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="75" spans="1:6">
+      <c r="G74" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7">
       <c r="A75" t="s">
         <v>273</v>
       </c>
@@ -4491,8 +5085,11 @@
       <c r="F75" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="76" spans="1:6">
+      <c r="G75" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7">
       <c r="A76" t="s">
         <v>276</v>
       </c>
@@ -4511,8 +5108,11 @@
       <c r="F76" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="77" spans="1:6">
+      <c r="G76" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7">
       <c r="A77" t="s">
         <v>280</v>
       </c>
@@ -4531,8 +5131,11 @@
       <c r="F77" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="78" spans="1:6">
+      <c r="G77" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
       <c r="A78" t="s">
         <v>284</v>
       </c>
@@ -4551,8 +5154,11 @@
       <c r="F78" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="79" spans="1:6">
+      <c r="G78" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7">
       <c r="A79" t="s">
         <v>288</v>
       </c>
@@ -4571,8 +5177,11 @@
       <c r="F79" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="80" spans="1:6">
+      <c r="G79" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7">
       <c r="A80" t="s">
         <v>291</v>
       </c>
@@ -4591,8 +5200,11 @@
       <c r="F80" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="81" spans="1:6">
+      <c r="G80" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7">
       <c r="A81" t="s">
         <v>294</v>
       </c>
@@ -4611,8 +5223,11 @@
       <c r="F81" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="82" spans="1:6">
+      <c r="G81" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7">
       <c r="A82" t="s">
         <v>298</v>
       </c>
@@ -4631,8 +5246,11 @@
       <c r="F82" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="83" spans="1:6">
+      <c r="G82" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
       <c r="A83" t="s">
         <v>302</v>
       </c>
@@ -4651,8 +5269,11 @@
       <c r="F83" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="84" spans="1:6">
+      <c r="G83" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
       <c r="A84" t="s">
         <v>306</v>
       </c>
@@ -4671,8 +5292,11 @@
       <c r="F84" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="85" spans="1:6">
+      <c r="G84" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
       <c r="A85" t="s">
         <v>309</v>
       </c>
@@ -4691,8 +5315,11 @@
       <c r="F85" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="86" spans="1:6">
+      <c r="G85" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
       <c r="A86" t="s">
         <v>312</v>
       </c>
@@ -4711,8 +5338,11 @@
       <c r="F86" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="87" spans="1:6">
+      <c r="G86" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7">
       <c r="A87" t="s">
         <v>316</v>
       </c>
@@ -4731,8 +5361,11 @@
       <c r="F87" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="88" spans="1:6">
+      <c r="G87" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7">
       <c r="A88" t="s">
         <v>320</v>
       </c>
@@ -4751,8 +5384,11 @@
       <c r="F88" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="89" spans="1:6">
+      <c r="G88" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7">
       <c r="A89" t="s">
         <v>324</v>
       </c>
@@ -4771,8 +5407,11 @@
       <c r="F89" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="90" spans="1:6">
+      <c r="G89" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
       <c r="A90" t="s">
         <v>327</v>
       </c>
@@ -4791,8 +5430,11 @@
       <c r="F90" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="91" spans="1:6">
+      <c r="G90" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7">
       <c r="A91" t="s">
         <v>330</v>
       </c>
@@ -4811,8 +5453,11 @@
       <c r="F91" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="92" spans="1:6">
+      <c r="G91" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
       <c r="A92" t="s">
         <v>334</v>
       </c>
@@ -4831,8 +5476,11 @@
       <c r="F92" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="93" spans="1:6">
+      <c r="G92" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7">
       <c r="A93" t="s">
         <v>338</v>
       </c>
@@ -4851,8 +5499,11 @@
       <c r="F93" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="94" spans="1:6">
+      <c r="G93" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7">
       <c r="A94" t="s">
         <v>342</v>
       </c>
@@ -4871,8 +5522,11 @@
       <c r="F94" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="95" spans="1:6">
+      <c r="G94" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7">
       <c r="A95" t="s">
         <v>345</v>
       </c>
@@ -4891,8 +5545,11 @@
       <c r="F95" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="96" spans="1:6">
+      <c r="G95" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7">
       <c r="A96" t="s">
         <v>348</v>
       </c>
@@ -4911,8 +5568,11 @@
       <c r="F96" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="97" spans="1:6">
+      <c r="G96" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7">
       <c r="A97" t="s">
         <v>352</v>
       </c>
@@ -4931,8 +5591,11 @@
       <c r="F97" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="98" spans="1:6">
+      <c r="G97" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7">
       <c r="A98" t="s">
         <v>356</v>
       </c>
@@ -4951,8 +5614,11 @@
       <c r="F98" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="99" spans="1:6">
+      <c r="G98" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7">
       <c r="A99" t="s">
         <v>360</v>
       </c>
@@ -4971,8 +5637,11 @@
       <c r="F99" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="100" spans="1:6">
+      <c r="G99" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7">
       <c r="A100" t="s">
         <v>363</v>
       </c>
@@ -4991,8 +5660,11 @@
       <c r="F100" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="101" spans="1:6">
+      <c r="G100" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7">
       <c r="A101" t="s">
         <v>366</v>
       </c>
@@ -5011,8 +5683,11 @@
       <c r="F101" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="102" spans="1:6">
+      <c r="G101" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7">
       <c r="A102" t="s">
         <v>370</v>
       </c>
@@ -5031,8 +5706,11 @@
       <c r="F102" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="103" spans="1:6">
+      <c r="G102" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7">
       <c r="A103" t="s">
         <v>374</v>
       </c>
@@ -5051,8 +5729,11 @@
       <c r="F103" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="104" spans="1:6">
+      <c r="G103" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7">
       <c r="A104" t="s">
         <v>377</v>
       </c>
@@ -5071,8 +5752,11 @@
       <c r="F104" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="105" spans="1:6">
+      <c r="G104" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7">
       <c r="A105" t="s">
         <v>380</v>
       </c>
@@ -5091,8 +5775,11 @@
       <c r="F105" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="106" spans="1:6">
+      <c r="G105" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7">
       <c r="A106" t="s">
         <v>383</v>
       </c>
@@ -5111,8 +5798,11 @@
       <c r="F106" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="107" spans="1:6">
+      <c r="G106" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7">
       <c r="A107" t="s">
         <v>387</v>
       </c>
@@ -5131,8 +5821,11 @@
       <c r="F107" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="108" spans="1:6">
+      <c r="G107" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7">
       <c r="A108" t="s">
         <v>391</v>
       </c>
@@ -5151,8 +5844,11 @@
       <c r="F108" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="109" spans="1:6">
+      <c r="G108" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7">
       <c r="A109" t="s">
         <v>395</v>
       </c>
@@ -5171,8 +5867,11 @@
       <c r="F109" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="110" spans="1:6">
+      <c r="G109" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7">
       <c r="A110" t="s">
         <v>398</v>
       </c>
@@ -5191,8 +5890,11 @@
       <c r="F110" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="111" spans="1:6">
+      <c r="G110" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7">
       <c r="A111" t="s">
         <v>401</v>
       </c>
@@ -5211,8 +5913,11 @@
       <c r="F111" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="112" spans="1:6">
+      <c r="G111" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7">
       <c r="A112" t="s">
         <v>405</v>
       </c>
@@ -5231,8 +5936,11 @@
       <c r="F112" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="113" spans="1:6">
+      <c r="G112" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7">
       <c r="A113" t="s">
         <v>409</v>
       </c>
@@ -5251,8 +5959,11 @@
       <c r="F113" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="114" spans="1:6">
+      <c r="G113" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7">
       <c r="A114" t="s">
         <v>413</v>
       </c>
@@ -5271,8 +5982,11 @@
       <c r="F114" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="115" spans="1:6">
+      <c r="G114" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7">
       <c r="A115" t="s">
         <v>416</v>
       </c>
@@ -5291,8 +6005,11 @@
       <c r="F115" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="116" spans="1:6">
+      <c r="G115" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7">
       <c r="A116" t="s">
         <v>419</v>
       </c>
@@ -5311,8 +6028,11 @@
       <c r="F116" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="117" spans="1:6">
+      <c r="G116" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7">
       <c r="A117" t="s">
         <v>422</v>
       </c>
@@ -5331,8 +6051,11 @@
       <c r="F117" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="118" spans="1:6">
+      <c r="G117" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7">
       <c r="A118" t="s">
         <v>425</v>
       </c>
@@ -5351,8 +6074,11 @@
       <c r="F118" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="119" spans="1:6">
+      <c r="G118" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7">
       <c r="A119" t="s">
         <v>429</v>
       </c>
@@ -5371,8 +6097,11 @@
       <c r="F119" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="120" spans="1:6">
+      <c r="G119" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7">
       <c r="A120" t="s">
         <v>432</v>
       </c>
@@ -5391,8 +6120,11 @@
       <c r="F120" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="121" spans="1:6">
+      <c r="G120" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7">
       <c r="A121" t="s">
         <v>435</v>
       </c>
@@ -5411,8 +6143,11 @@
       <c r="F121" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="122" spans="1:6">
+      <c r="G121" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7">
       <c r="A122" t="s">
         <v>438</v>
       </c>
@@ -5431,8 +6166,11 @@
       <c r="F122" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="123" spans="1:6">
+      <c r="G122" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7">
       <c r="A123" t="s">
         <v>441</v>
       </c>
@@ -5451,8 +6189,11 @@
       <c r="F123" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="124" spans="1:6">
+      <c r="G123" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7">
       <c r="A124" t="s">
         <v>445</v>
       </c>
@@ -5471,8 +6212,11 @@
       <c r="F124" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="125" spans="1:6">
+      <c r="G124" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7">
       <c r="A125" t="s">
         <v>447</v>
       </c>
@@ -5491,8 +6235,11 @@
       <c r="F125" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="126" spans="1:6">
+      <c r="G125" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7">
       <c r="A126" t="s">
         <v>450</v>
       </c>
@@ -5511,8 +6258,11 @@
       <c r="F126" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="127" spans="1:6">
+      <c r="G126" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7">
       <c r="A127" t="s">
         <v>453</v>
       </c>
@@ -5531,8 +6281,11 @@
       <c r="F127" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="128" spans="1:6">
+      <c r="G127" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7">
       <c r="A128" t="s">
         <v>456</v>
       </c>
@@ -5551,8 +6304,11 @@
       <c r="F128" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="129" spans="1:6">
+      <c r="G128" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7">
       <c r="A129" t="s">
         <v>460</v>
       </c>
@@ -5571,8 +6327,11 @@
       <c r="F129" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="130" spans="1:6">
+      <c r="G129" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7">
       <c r="A130" t="s">
         <v>463</v>
       </c>
@@ -5591,8 +6350,11 @@
       <c r="F130" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="131" spans="1:6">
+      <c r="G130" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7">
       <c r="A131" t="s">
         <v>466</v>
       </c>
@@ -5611,8 +6373,11 @@
       <c r="F131" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="132" spans="1:6">
+      <c r="G131" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7">
       <c r="A132" t="s">
         <v>469</v>
       </c>
@@ -5631,8 +6396,11 @@
       <c r="F132" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="133" spans="1:6">
+      <c r="G132" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7">
       <c r="A133" t="s">
         <v>472</v>
       </c>
@@ -5651,8 +6419,11 @@
       <c r="F133" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="134" spans="1:6">
+      <c r="G133" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7">
       <c r="A134" t="s">
         <v>476</v>
       </c>
@@ -5670,6 +6441,9 @@
       </c>
       <c r="F134" t="s">
         <v>73</v>
+      </c>
+      <c r="G134" t="s">
+        <v>1031</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(excel): expand complex showcase templates
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Core.xlsx
+++ b/examples/showcase/data/Core.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Item" sheetId="1" r:id="rId1"/>
     <sheet name="GameSettings" sheetId="2" r:id="rId2"/>
-    <sheet name="Localization" sheetId="3" r:id="rId3"/>
-    <sheet name="LevelExp" sheetId="4" r:id="rId4"/>
+    <sheet name="MaintenanceWindow" sheetId="3" r:id="rId3"/>
+    <sheet name="Localization" sheetId="4" r:id="rId4"/>
+    <sheet name="LevelExp" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47,8 +48,7 @@
 Field: id
 Type: i32
 Scope: all
-Key: yes
-Required: yes</t>
+Key: yes</t>
         </r>
       </text>
     </comment>
@@ -76,7 +76,6 @@
 Field: name
 Type: string
 Scope: all
-Required: yes
 Length: 2..32</t>
         </r>
       </text>
@@ -104,8 +103,7 @@
 Item category
 Field: item_type
 Type: enum&lt;ItemType&gt;
-Scope: all
-Required: yes</t>
+Scope: all</t>
         </r>
       </text>
     </comment>
@@ -163,7 +161,7 @@
 Type: struct&lt;ResourceCost&gt;
 Scope: all
 Tuple fields: kind: enum&lt;ResourceKind&gt;, id: i32, count: i32
-Required: yes</t>
+Parser: tuple</t>
         </r>
       </text>
     </comment>
@@ -192,6 +190,7 @@
 Type: set&lt;string&gt;
 Scope: all
 Default: ["misc"]
+Parser: json
 Length: 1..5</t>
         </r>
       </text>
@@ -220,7 +219,7 @@
 Field: attributes
 Type: map&lt;string,i32&gt;
 Scope: all
-Required: yes</t>
+Parser: map</t>
         </r>
       </text>
     </comment>
@@ -259,7 +258,120 @@
 Type: struct&lt;Vec3&gt;
 Scope: all
 Tuple fields: x: f32, y: f32, z: f32
-Required: yes</t>
+Parser: tuple</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Double precision tuning value
+Field: gravity
+Type: f64
+Scope: all</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Fixed-length array parsed from one cell
+Field: daily_bonus_items
+Type: array&lt;ref&lt;Item.id&gt;,3&gt;
+Scope: all
+Parser: split</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Fixed-length array of structs
+Field: spawn_points
+Type: array&lt;struct&lt;Vec3&gt;,2&gt;
+Scope: all
+Tuple fields: x: f32, y: f32, z: f32
+Parser: tuple_list</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Optional derived struct copied from a child row
+Field: maintenance
+Type: optional&lt;struct&lt;MaintenanceInfo&gt;&gt;
+Scope: all
+Generated: yes; do not fill this column.
+From: MaintenanceWindow.version -&gt; version</t>
         </r>
       </text>
     </comment>
@@ -268,7 +380,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="1029">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="1057">
   <si>
     <t>@table</t>
   </si>
@@ -348,25 +460,25 @@
     <t>#scope</t>
   </si>
   <si>
-    <t>#rule</t>
+    <t>#input</t>
   </si>
   <si>
     <t>key</t>
   </si>
   <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>optional;range=1..9999</t>
-  </si>
-  <si>
-    <t>required;parser=tuple</t>
-  </si>
-  <si>
-    <t>optional;parser=json</t>
-  </si>
-  <si>
-    <t>required;parser=map</t>
+    <t>length=2..32</t>
+  </si>
+  <si>
+    <t>range=1..9999</t>
+  </si>
+  <si>
+    <t>parser=tuple</t>
+  </si>
+  <si>
+    <t>parser=json;length=1..5</t>
+  </si>
+  <si>
+    <t>parser=map</t>
   </si>
   <si>
     <t>#desc</t>
@@ -2091,7 +2203,7 @@
     <t>singleton</t>
   </si>
   <si>
-    <t>c12bf4c9c7ee2403</t>
+    <t>45bbcde237c37a75</t>
   </si>
   <si>
     <t>version</t>
@@ -2109,16 +2221,64 @@
     <t>starter_items</t>
   </si>
   <si>
+    <t>gravity</t>
+  </si>
+  <si>
+    <t>daily_bonus_items</t>
+  </si>
+  <si>
+    <t>spawn_points</t>
+  </si>
+  <si>
+    <t>maintenance</t>
+  </si>
+  <si>
     <t>struct&lt;Vec3&gt;(x: f32, y: f32, z: f32)</t>
   </si>
   <si>
     <t>list&lt;ref&lt;Item.id&gt;&gt;</t>
   </si>
   <si>
-    <t>required;range=0..23</t>
-  </si>
-  <si>
-    <t>optional;range=0..999999</t>
+    <t>f64</t>
+  </si>
+  <si>
+    <t>array&lt;ref&lt;Item.id&gt;,3&gt;</t>
+  </si>
+  <si>
+    <t>array&lt;struct&lt;Vec3&gt;,2&gt;(x: f32, y: f32, z: f32)</t>
+  </si>
+  <si>
+    <t>optional&lt;struct&lt;MaintenanceInfo&gt;&gt;</t>
+  </si>
+  <si>
+    <t>range=0..23</t>
+  </si>
+  <si>
+    <t>range=0..999999</t>
+  </si>
+  <si>
+    <t>parser=json;length=1..4</t>
+  </si>
+  <si>
+    <t>parser=split</t>
+  </si>
+  <si>
+    <t>parser=tuple_list</t>
+  </si>
+  <si>
+    <t>from=MaintenanceWindow;match=version-&gt;version</t>
+  </si>
+  <si>
+    <t>Double precision tuning value</t>
+  </si>
+  <si>
+    <t>Fixed-length array parsed from one cell</t>
+  </si>
+  <si>
+    <t>Fixed-length array of structs</t>
+  </si>
+  <si>
+    <t>Optional derived struct copied from a child row Generated from MaintenanceWindow; do not fill this column.</t>
   </si>
   <si>
     <t>2026.05</t>
@@ -2130,6 +2290,45 @@
     <t>[1001,2001]</t>
   </si>
   <si>
+    <t>9.80665</t>
+  </si>
+  <si>
+    <t>1001,1002,2001</t>
+  </si>
+  <si>
+    <t>0,0,0|12,0,8</t>
+  </si>
+  <si>
+    <t>MaintenanceWindow</t>
+  </si>
+  <si>
+    <t>list</t>
+  </si>
+  <si>
+    <t>015c515a2f334276</t>
+  </si>
+  <si>
+    <t>starts_at</t>
+  </si>
+  <si>
+    <t>duration_minutes</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>optional&lt;string&gt;</t>
+  </si>
+  <si>
+    <t>range=1..1440</t>
+  </si>
+  <si>
+    <t>2026-06-01T03:00:00Z</t>
+  </si>
+  <si>
+    <t>Season rollout</t>
+  </si>
+  <si>
     <t>Localization</t>
   </si>
   <si>
@@ -2145,10 +2344,7 @@
     <t>note</t>
   </si>
   <si>
-    <t>optional&lt;string&gt;</t>
-  </si>
-  <si>
-    <t>optional</t>
+    <t>key;length=3..64</t>
   </si>
   <si>
     <t>loc_001</t>
@@ -2916,7 +3112,7 @@
     <t>key;range=1..100</t>
   </si>
   <si>
-    <t>required;range=0..999999999</t>
+    <t>range=0..999999999</t>
   </si>
   <si>
     <t>100</t>
@@ -3361,7 +3557,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3386,13 +3582,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="8"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3435,6 +3639,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE5E7EB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -3463,7 +3673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3482,6 +3692,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3783,8 +3996,7 @@
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="32.7109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" style="5" customWidth="1"/>
+    <col min="5" max="6" width="32.7109375" style="5" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" style="5" customWidth="1"/>
     <col min="8" max="8" width="30.7109375" style="5" customWidth="1"/>
   </cols>
@@ -3935,9 +4147,7 @@
       <c r="C6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
         <v>29</v>
       </c>
@@ -6805,8 +7015,11 @@
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="29.7109375" style="5" customWidth="1"/>
+    <col min="8" max="9" width="32.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="32.7109375" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -6835,10 +7048,8 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>fc4147b34b18d1d8</t>
-        </is>
+      <c r="J1" s="2" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6860,6 +7071,18 @@
       <c r="F2" s="3" t="s">
         <v>612</v>
       </c>
+      <c r="G2" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>616</v>
+      </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
@@ -6880,6 +7103,18 @@
       <c r="F3" s="5" t="s">
         <v>612</v>
       </c>
+      <c r="G3" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>616</v>
+      </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
@@ -6895,10 +7130,22 @@
         <v>19</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>614</v>
+        <v>618</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -6920,27 +7167,45 @@
       <c r="F5" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>required;parser=json</t>
-        </is>
+      <c r="F6" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>628</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
@@ -6952,20 +7217,44 @@
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>632</v>
+      </c>
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="5" t="s">
-        <v>617</v>
+        <v>633</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>487</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>618</v>
+        <v>634</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>619</v>
+        <v>635</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>636</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>637</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>628</v>
       </c>
     </row>
   </sheetData>
@@ -6985,7 +7274,160 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="5" width="16.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2"/>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>608</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>642</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5" t="s">
+        <v>646</v>
+      </c>
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="B8" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>647</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>648</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 1440." promptTitle="Integer range" prompt="Enter an integer from 1 to 1440." sqref="D8:D1007">
+      <formula1>1</formula1>
+      <formula2>1440</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -6999,7 +7441,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>620</v>
+        <v>649</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7023,7 +7465,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>621</v>
+        <v>650</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7034,13 +7476,13 @@
         <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>622</v>
+        <v>651</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>623</v>
+        <v>652</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>624</v>
+        <v>653</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -7051,13 +7493,13 @@
         <v>27</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>622</v>
+        <v>651</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>623</v>
+        <v>652</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>624</v>
+        <v>653</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -7074,7 +7516,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>625</v>
+        <v>645</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -7099,17 +7541,11 @@
         <v>26</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>626</v>
-      </c>
+        <v>654</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -7122,978 +7558,978 @@
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="5" t="s">
-        <v>627</v>
+        <v>655</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>628</v>
+        <v>656</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>629</v>
+        <v>657</v>
       </c>
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="5" t="s">
-        <v>630</v>
+        <v>658</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>631</v>
+        <v>659</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>632</v>
+        <v>660</v>
       </c>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:10">
       <c r="B10" s="5" t="s">
-        <v>633</v>
+        <v>661</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>634</v>
+        <v>662</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>635</v>
+        <v>663</v>
       </c>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:10">
       <c r="B11" s="5" t="s">
-        <v>636</v>
+        <v>664</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>637</v>
+        <v>665</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>638</v>
+        <v>666</v>
       </c>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:10">
       <c r="B12" s="5" t="s">
-        <v>639</v>
+        <v>667</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>640</v>
+        <v>668</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>641</v>
+        <v>669</v>
       </c>
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:10">
       <c r="B13" s="5" t="s">
-        <v>642</v>
+        <v>670</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>643</v>
+        <v>671</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>644</v>
+        <v>672</v>
       </c>
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:10">
       <c r="B14" s="5" t="s">
-        <v>645</v>
+        <v>673</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>646</v>
+        <v>674</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>647</v>
+        <v>675</v>
       </c>
       <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:10">
       <c r="B15" s="5" t="s">
-        <v>648</v>
+        <v>676</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>649</v>
+        <v>677</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>650</v>
+        <v>678</v>
       </c>
       <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:10">
       <c r="B16" s="5" t="s">
-        <v>651</v>
+        <v>679</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>652</v>
+        <v>680</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>653</v>
+        <v>681</v>
       </c>
       <c r="E16" s="5"/>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="5" t="s">
-        <v>654</v>
+        <v>682</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>655</v>
+        <v>683</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>656</v>
+        <v>684</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>657</v>
+        <v>685</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="5" t="s">
-        <v>658</v>
+        <v>686</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>659</v>
+        <v>687</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>660</v>
+        <v>688</v>
       </c>
       <c r="E18" s="5"/>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="5" t="s">
-        <v>661</v>
+        <v>689</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>662</v>
+        <v>690</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>663</v>
+        <v>691</v>
       </c>
       <c r="E19" s="5"/>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="5" t="s">
-        <v>664</v>
+        <v>692</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>665</v>
+        <v>693</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>666</v>
+        <v>694</v>
       </c>
       <c r="E20" s="5"/>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="5" t="s">
-        <v>667</v>
+        <v>695</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>668</v>
+        <v>696</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>669</v>
+        <v>697</v>
       </c>
       <c r="E21" s="5"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="5" t="s">
-        <v>670</v>
+        <v>698</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>671</v>
+        <v>699</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>672</v>
+        <v>700</v>
       </c>
       <c r="E22" s="5"/>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="5" t="s">
-        <v>673</v>
+        <v>701</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>674</v>
+        <v>702</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>675</v>
+        <v>703</v>
       </c>
       <c r="E23" s="5"/>
     </row>
     <row r="24" spans="2:5">
       <c r="B24" s="5" t="s">
-        <v>676</v>
+        <v>704</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>677</v>
+        <v>705</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>678</v>
+        <v>706</v>
       </c>
       <c r="E24" s="5"/>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="5" t="s">
-        <v>679</v>
+        <v>707</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>680</v>
+        <v>708</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>681</v>
+        <v>709</v>
       </c>
       <c r="E25" s="5"/>
     </row>
     <row r="26" spans="2:5">
       <c r="B26" s="5" t="s">
-        <v>682</v>
+        <v>710</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>683</v>
+        <v>711</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>684</v>
+        <v>712</v>
       </c>
       <c r="E26" s="5"/>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="5" t="s">
-        <v>685</v>
+        <v>713</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>686</v>
+        <v>714</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>687</v>
+        <v>715</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>688</v>
+        <v>716</v>
       </c>
     </row>
     <row r="28" spans="2:5">
       <c r="B28" s="5" t="s">
-        <v>689</v>
+        <v>717</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>690</v>
+        <v>718</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>691</v>
+        <v>719</v>
       </c>
       <c r="E28" s="5"/>
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="5" t="s">
-        <v>692</v>
+        <v>720</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>693</v>
+        <v>721</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>694</v>
+        <v>722</v>
       </c>
       <c r="E29" s="5"/>
     </row>
     <row r="30" spans="2:5">
       <c r="B30" s="5" t="s">
-        <v>695</v>
+        <v>723</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>696</v>
+        <v>724</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>697</v>
+        <v>725</v>
       </c>
       <c r="E30" s="5"/>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="5" t="s">
-        <v>698</v>
+        <v>726</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>699</v>
+        <v>727</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>700</v>
+        <v>728</v>
       </c>
       <c r="E31" s="5"/>
     </row>
     <row r="32" spans="2:5">
       <c r="B32" s="5" t="s">
-        <v>701</v>
+        <v>729</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>702</v>
+        <v>730</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>703</v>
+        <v>731</v>
       </c>
       <c r="E32" s="5"/>
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="5" t="s">
-        <v>704</v>
+        <v>732</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>705</v>
+        <v>733</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>706</v>
+        <v>734</v>
       </c>
       <c r="E33" s="5"/>
     </row>
     <row r="34" spans="2:5">
       <c r="B34" s="5" t="s">
-        <v>707</v>
+        <v>735</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>708</v>
+        <v>736</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>709</v>
+        <v>737</v>
       </c>
       <c r="E34" s="5"/>
     </row>
     <row r="35" spans="2:5">
       <c r="B35" s="5" t="s">
-        <v>710</v>
+        <v>738</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>711</v>
+        <v>739</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>712</v>
+        <v>740</v>
       </c>
       <c r="E35" s="5"/>
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="5" t="s">
-        <v>713</v>
+        <v>741</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>714</v>
+        <v>742</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>715</v>
+        <v>743</v>
       </c>
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="5" t="s">
-        <v>716</v>
+        <v>744</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>717</v>
+        <v>745</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>718</v>
+        <v>746</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>719</v>
+        <v>747</v>
       </c>
     </row>
     <row r="38" spans="2:5">
       <c r="B38" s="5" t="s">
-        <v>720</v>
+        <v>748</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>721</v>
+        <v>749</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>722</v>
+        <v>750</v>
       </c>
       <c r="E38" s="5"/>
     </row>
     <row r="39" spans="2:5">
       <c r="B39" s="5" t="s">
-        <v>723</v>
+        <v>751</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>724</v>
+        <v>752</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>725</v>
+        <v>753</v>
       </c>
       <c r="E39" s="5"/>
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="5" t="s">
-        <v>726</v>
+        <v>754</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>727</v>
+        <v>755</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>728</v>
+        <v>756</v>
       </c>
       <c r="E40" s="5"/>
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="5" t="s">
-        <v>729</v>
+        <v>757</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>730</v>
+        <v>758</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>731</v>
+        <v>759</v>
       </c>
       <c r="E41" s="5"/>
     </row>
     <row r="42" spans="2:5">
       <c r="B42" s="5" t="s">
-        <v>732</v>
+        <v>760</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>733</v>
+        <v>761</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>734</v>
+        <v>762</v>
       </c>
       <c r="E42" s="5"/>
     </row>
     <row r="43" spans="2:5">
       <c r="B43" s="5" t="s">
-        <v>735</v>
+        <v>763</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>736</v>
+        <v>764</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>737</v>
+        <v>765</v>
       </c>
       <c r="E43" s="5"/>
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="5" t="s">
-        <v>738</v>
+        <v>766</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>739</v>
+        <v>767</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>740</v>
+        <v>768</v>
       </c>
       <c r="E44" s="5"/>
     </row>
     <row r="45" spans="2:5">
       <c r="B45" s="5" t="s">
-        <v>741</v>
+        <v>769</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>742</v>
+        <v>770</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>743</v>
+        <v>771</v>
       </c>
       <c r="E45" s="5"/>
     </row>
     <row r="46" spans="2:5">
       <c r="B46" s="5" t="s">
-        <v>744</v>
+        <v>772</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>745</v>
+        <v>773</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>746</v>
+        <v>774</v>
       </c>
       <c r="E46" s="5"/>
     </row>
     <row r="47" spans="2:5">
       <c r="B47" s="5" t="s">
-        <v>747</v>
+        <v>775</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>748</v>
+        <v>776</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>749</v>
+        <v>777</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>750</v>
+        <v>778</v>
       </c>
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="5" t="s">
-        <v>751</v>
+        <v>779</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>752</v>
+        <v>780</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>753</v>
+        <v>781</v>
       </c>
       <c r="E48" s="5"/>
     </row>
     <row r="49" spans="2:5">
       <c r="B49" s="5" t="s">
-        <v>754</v>
+        <v>782</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>755</v>
+        <v>783</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>756</v>
+        <v>784</v>
       </c>
       <c r="E49" s="5"/>
     </row>
     <row r="50" spans="2:5">
       <c r="B50" s="5" t="s">
-        <v>757</v>
+        <v>785</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>758</v>
+        <v>786</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>759</v>
+        <v>787</v>
       </c>
       <c r="E50" s="5"/>
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="5" t="s">
-        <v>760</v>
+        <v>788</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>761</v>
+        <v>789</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>762</v>
+        <v>790</v>
       </c>
       <c r="E51" s="5"/>
     </row>
     <row r="52" spans="2:5">
       <c r="B52" s="5" t="s">
-        <v>763</v>
+        <v>791</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>764</v>
+        <v>792</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>765</v>
+        <v>793</v>
       </c>
       <c r="E52" s="5"/>
     </row>
     <row r="53" spans="2:5">
       <c r="B53" s="5" t="s">
-        <v>766</v>
+        <v>794</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>767</v>
+        <v>795</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>768</v>
+        <v>796</v>
       </c>
       <c r="E53" s="5"/>
     </row>
     <row r="54" spans="2:5">
       <c r="B54" s="5" t="s">
-        <v>769</v>
+        <v>797</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>770</v>
+        <v>798</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>771</v>
+        <v>799</v>
       </c>
       <c r="E54" s="5"/>
     </row>
     <row r="55" spans="2:5">
       <c r="B55" s="5" t="s">
-        <v>772</v>
+        <v>800</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>773</v>
+        <v>801</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>774</v>
+        <v>802</v>
       </c>
       <c r="E55" s="5"/>
     </row>
     <row r="56" spans="2:5">
       <c r="B56" s="5" t="s">
-        <v>775</v>
+        <v>803</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>776</v>
+        <v>804</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>777</v>
+        <v>805</v>
       </c>
       <c r="E56" s="5"/>
     </row>
     <row r="57" spans="2:5">
       <c r="B57" s="5" t="s">
-        <v>778</v>
+        <v>806</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>779</v>
+        <v>807</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>780</v>
+        <v>808</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>781</v>
+        <v>809</v>
       </c>
     </row>
     <row r="58" spans="2:5">
       <c r="B58" s="5" t="s">
-        <v>782</v>
+        <v>810</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>783</v>
+        <v>811</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>784</v>
+        <v>812</v>
       </c>
       <c r="E58" s="5"/>
     </row>
     <row r="59" spans="2:5">
       <c r="B59" s="5" t="s">
-        <v>785</v>
+        <v>813</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>786</v>
+        <v>814</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>787</v>
+        <v>815</v>
       </c>
       <c r="E59" s="5"/>
     </row>
     <row r="60" spans="2:5">
       <c r="B60" s="5" t="s">
-        <v>788</v>
+        <v>816</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>789</v>
+        <v>817</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>790</v>
+        <v>818</v>
       </c>
       <c r="E60" s="5"/>
     </row>
     <row r="61" spans="2:5">
       <c r="B61" s="5" t="s">
-        <v>791</v>
+        <v>819</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>792</v>
+        <v>820</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>793</v>
+        <v>821</v>
       </c>
       <c r="E61" s="5"/>
     </row>
     <row r="62" spans="2:5">
       <c r="B62" s="5" t="s">
-        <v>794</v>
+        <v>822</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>795</v>
+        <v>823</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>796</v>
+        <v>824</v>
       </c>
       <c r="E62" s="5"/>
     </row>
     <row r="63" spans="2:5">
       <c r="B63" s="5" t="s">
-        <v>797</v>
+        <v>825</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>798</v>
+        <v>826</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>799</v>
+        <v>827</v>
       </c>
       <c r="E63" s="5"/>
     </row>
     <row r="64" spans="2:5">
       <c r="B64" s="5" t="s">
-        <v>800</v>
+        <v>828</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>801</v>
+        <v>829</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>802</v>
+        <v>830</v>
       </c>
       <c r="E64" s="5"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="5" t="s">
-        <v>803</v>
+        <v>831</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>804</v>
+        <v>832</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>805</v>
+        <v>833</v>
       </c>
       <c r="E65" s="5"/>
     </row>
     <row r="66" spans="2:5">
       <c r="B66" s="5" t="s">
-        <v>806</v>
+        <v>834</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>807</v>
+        <v>835</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>808</v>
+        <v>836</v>
       </c>
       <c r="E66" s="5"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="5" t="s">
-        <v>809</v>
+        <v>837</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>810</v>
+        <v>838</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>811</v>
+        <v>839</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>812</v>
+        <v>840</v>
       </c>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="5" t="s">
-        <v>813</v>
+        <v>841</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>814</v>
+        <v>842</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>815</v>
+        <v>843</v>
       </c>
       <c r="E68" s="5"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="5" t="s">
-        <v>816</v>
+        <v>844</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>817</v>
+        <v>845</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>818</v>
+        <v>846</v>
       </c>
       <c r="E69" s="5"/>
     </row>
     <row r="70" spans="2:5">
       <c r="B70" s="5" t="s">
-        <v>819</v>
+        <v>847</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>820</v>
+        <v>848</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>821</v>
+        <v>849</v>
       </c>
       <c r="E70" s="5"/>
     </row>
     <row r="71" spans="2:5">
       <c r="B71" s="5" t="s">
-        <v>822</v>
+        <v>850</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>823</v>
+        <v>851</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>824</v>
+        <v>852</v>
       </c>
       <c r="E71" s="5"/>
     </row>
     <row r="72" spans="2:5">
       <c r="B72" s="5" t="s">
-        <v>825</v>
+        <v>853</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>826</v>
+        <v>854</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>827</v>
+        <v>855</v>
       </c>
       <c r="E72" s="5"/>
     </row>
     <row r="73" spans="2:5">
       <c r="B73" s="5" t="s">
-        <v>828</v>
+        <v>856</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>829</v>
+        <v>857</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>830</v>
+        <v>858</v>
       </c>
       <c r="E73" s="5"/>
     </row>
     <row r="74" spans="2:5">
       <c r="B74" s="5" t="s">
-        <v>831</v>
+        <v>859</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>832</v>
+        <v>860</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>833</v>
+        <v>861</v>
       </c>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="2:5">
       <c r="B75" s="5" t="s">
-        <v>834</v>
+        <v>862</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>835</v>
+        <v>863</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>836</v>
+        <v>864</v>
       </c>
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="2:5">
       <c r="B76" s="5" t="s">
-        <v>837</v>
+        <v>865</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>838</v>
+        <v>866</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>839</v>
+        <v>867</v>
       </c>
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="2:5">
       <c r="B77" s="5" t="s">
-        <v>840</v>
+        <v>868</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>841</v>
+        <v>869</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>842</v>
+        <v>870</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>843</v>
+        <v>871</v>
       </c>
     </row>
     <row r="78" spans="2:5">
       <c r="B78" s="5" t="s">
-        <v>844</v>
+        <v>872</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>845</v>
+        <v>873</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>846</v>
+        <v>874</v>
       </c>
       <c r="E78" s="5"/>
     </row>
     <row r="79" spans="2:5">
       <c r="B79" s="5" t="s">
-        <v>847</v>
+        <v>875</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>848</v>
+        <v>876</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>849</v>
+        <v>877</v>
       </c>
       <c r="E79" s="5"/>
     </row>
     <row r="80" spans="2:5">
       <c r="B80" s="5" t="s">
-        <v>850</v>
+        <v>878</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>851</v>
+        <v>879</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>852</v>
+        <v>880</v>
       </c>
       <c r="E80" s="5"/>
     </row>
     <row r="81" spans="2:5">
       <c r="B81" s="5" t="s">
-        <v>853</v>
+        <v>881</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>854</v>
+        <v>882</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>855</v>
+        <v>883</v>
       </c>
       <c r="E81" s="5"/>
     </row>
     <row r="82" spans="2:5">
       <c r="B82" s="5" t="s">
-        <v>856</v>
+        <v>884</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>857</v>
+        <v>885</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>858</v>
+        <v>886</v>
       </c>
       <c r="E82" s="5"/>
     </row>
     <row r="83" spans="2:5">
       <c r="B83" s="5" t="s">
-        <v>859</v>
+        <v>887</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>860</v>
+        <v>888</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>861</v>
+        <v>889</v>
       </c>
       <c r="E83" s="5"/>
     </row>
     <row r="84" spans="2:5">
       <c r="B84" s="5" t="s">
-        <v>862</v>
+        <v>890</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>863</v>
+        <v>891</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>864</v>
+        <v>892</v>
       </c>
       <c r="E84" s="5"/>
     </row>
     <row r="85" spans="2:5">
       <c r="B85" s="5" t="s">
-        <v>865</v>
+        <v>893</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>866</v>
+        <v>894</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>867</v>
+        <v>895</v>
       </c>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="2:5">
       <c r="B86" s="5" t="s">
-        <v>868</v>
+        <v>896</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>869</v>
+        <v>897</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>870</v>
+        <v>898</v>
       </c>
       <c r="E86" s="5"/>
     </row>
     <row r="87" spans="2:5">
       <c r="B87" s="5" t="s">
-        <v>871</v>
+        <v>899</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>872</v>
+        <v>900</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>873</v>
+        <v>901</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>874</v>
+        <v>902</v>
       </c>
     </row>
   </sheetData>
@@ -8101,8 +8537,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -8116,7 +8552,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>875</v>
+        <v>903</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8128,7 +8564,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>876</v>
+        <v>904</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -8140,7 +8576,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>877</v>
+        <v>905</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -8148,13 +8584,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>876</v>
+        <v>904</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>878</v>
+        <v>906</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>879</v>
+        <v>907</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -8162,13 +8598,13 @@
         <v>17</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>876</v>
+        <v>904</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>878</v>
+        <v>906</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>879</v>
+        <v>907</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -8179,10 +8615,10 @@
         <v>19</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>880</v>
+        <v>908</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>625</v>
+        <v>645</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -8204,14 +8640,12 @@
         <v>26</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>881</v>
+        <v>909</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>882</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>626</v>
-      </c>
+        <v>910</v>
+      </c>
+      <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -8226,25 +8660,25 @@
         <v>44</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>883</v>
+        <v>911</v>
       </c>
       <c r="D8" s="5"/>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="5" t="s">
-        <v>884</v>
+        <v>912</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>885</v>
+        <v>913</v>
       </c>
       <c r="D9" s="5"/>
     </row>
     <row r="10" spans="1:10">
       <c r="B10" s="5" t="s">
-        <v>886</v>
+        <v>914</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>887</v>
+        <v>915</v>
       </c>
       <c r="D10" s="5"/>
     </row>
@@ -8253,7 +8687,7 @@
         <v>482</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>888</v>
+        <v>916</v>
       </c>
       <c r="D11" s="5"/>
     </row>
@@ -8262,7 +8696,7 @@
         <v>487</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>889</v>
+        <v>917</v>
       </c>
       <c r="D12" s="5"/>
     </row>
@@ -8271,25 +8705,25 @@
         <v>492</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>890</v>
+        <v>918</v>
       </c>
       <c r="D13" s="5"/>
     </row>
     <row r="14" spans="1:10">
       <c r="B14" s="5" t="s">
-        <v>891</v>
+        <v>919</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>892</v>
+        <v>920</v>
       </c>
       <c r="D14" s="5"/>
     </row>
     <row r="15" spans="1:10">
       <c r="B15" s="5" t="s">
-        <v>893</v>
+        <v>921</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>894</v>
+        <v>922</v>
       </c>
       <c r="D15" s="5"/>
     </row>
@@ -8298,7 +8732,7 @@
         <v>505</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>895</v>
+        <v>923</v>
       </c>
       <c r="D16" s="5"/>
     </row>
@@ -8307,10 +8741,10 @@
         <v>510</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>896</v>
+        <v>924</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>897</v>
+        <v>925</v>
       </c>
     </row>
     <row r="18" spans="2:4">
@@ -8318,25 +8752,25 @@
         <v>515</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>898</v>
+        <v>926</v>
       </c>
       <c r="D18" s="5"/>
     </row>
     <row r="19" spans="2:4">
       <c r="B19" s="5" t="s">
-        <v>899</v>
+        <v>927</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>900</v>
+        <v>928</v>
       </c>
       <c r="D19" s="5"/>
     </row>
     <row r="20" spans="2:4">
       <c r="B20" s="5" t="s">
-        <v>901</v>
+        <v>929</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>902</v>
+        <v>930</v>
       </c>
       <c r="D20" s="5"/>
     </row>
@@ -8345,7 +8779,7 @@
         <v>70</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>903</v>
+        <v>931</v>
       </c>
       <c r="D21" s="5"/>
     </row>
@@ -8354,7 +8788,7 @@
         <v>76</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>904</v>
+        <v>932</v>
       </c>
       <c r="D22" s="5"/>
     </row>
@@ -8363,16 +8797,16 @@
         <v>536</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>905</v>
+        <v>933</v>
       </c>
       <c r="D23" s="5"/>
     </row>
     <row r="24" spans="2:4">
       <c r="B24" s="5" t="s">
-        <v>906</v>
+        <v>934</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>907</v>
+        <v>935</v>
       </c>
       <c r="D24" s="5"/>
     </row>
@@ -8381,7 +8815,7 @@
         <v>93</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>908</v>
+        <v>936</v>
       </c>
       <c r="D25" s="5"/>
     </row>
@@ -8390,7 +8824,7 @@
         <v>99</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>909</v>
+        <v>937</v>
       </c>
       <c r="D26" s="5"/>
     </row>
@@ -8399,10 +8833,10 @@
         <v>104</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>910</v>
+        <v>938</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>911</v>
+        <v>939</v>
       </c>
     </row>
     <row r="28" spans="2:4">
@@ -8410,16 +8844,16 @@
         <v>557</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>912</v>
+        <v>940</v>
       </c>
       <c r="D28" s="5"/>
     </row>
     <row r="29" spans="2:4">
       <c r="B29" s="5" t="s">
-        <v>913</v>
+        <v>941</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>914</v>
+        <v>942</v>
       </c>
       <c r="D29" s="5"/>
     </row>
@@ -8428,7 +8862,7 @@
         <v>117</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>915</v>
+        <v>943</v>
       </c>
       <c r="D30" s="5"/>
     </row>
@@ -8437,7 +8871,7 @@
         <v>122</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>916</v>
+        <v>944</v>
       </c>
       <c r="D31" s="5"/>
     </row>
@@ -8446,7 +8880,7 @@
         <v>127</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>917</v>
+        <v>945</v>
       </c>
       <c r="D32" s="5"/>
     </row>
@@ -8455,16 +8889,16 @@
         <v>577</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>918</v>
+        <v>946</v>
       </c>
       <c r="D33" s="5"/>
     </row>
     <row r="34" spans="2:4">
       <c r="B34" s="5" t="s">
-        <v>919</v>
+        <v>947</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>920</v>
+        <v>948</v>
       </c>
       <c r="D34" s="5"/>
     </row>
@@ -8473,7 +8907,7 @@
         <v>139</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>921</v>
+        <v>949</v>
       </c>
       <c r="D35" s="5"/>
     </row>
@@ -8482,7 +8916,7 @@
         <v>144</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>922</v>
+        <v>950</v>
       </c>
       <c r="D36" s="5"/>
     </row>
@@ -8491,10 +8925,10 @@
         <v>149</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>923</v>
+        <v>951</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>924</v>
+        <v>952</v>
       </c>
     </row>
     <row r="38" spans="2:4">
@@ -8502,16 +8936,16 @@
         <v>598</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>925</v>
+        <v>953</v>
       </c>
       <c r="D38" s="5"/>
     </row>
     <row r="39" spans="2:4">
       <c r="B39" s="5" t="s">
-        <v>926</v>
+        <v>954</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>927</v>
+        <v>955</v>
       </c>
       <c r="D39" s="5"/>
     </row>
@@ -8520,7 +8954,7 @@
         <v>162</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>928</v>
+        <v>956</v>
       </c>
       <c r="D40" s="5"/>
     </row>
@@ -8529,7 +8963,7 @@
         <v>167</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>929</v>
+        <v>957</v>
       </c>
       <c r="D41" s="5"/>
     </row>
@@ -8538,25 +8972,25 @@
         <v>172</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>930</v>
+        <v>958</v>
       </c>
       <c r="D42" s="5"/>
     </row>
     <row r="43" spans="2:4">
       <c r="B43" s="5" t="s">
-        <v>931</v>
+        <v>959</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>932</v>
+        <v>960</v>
       </c>
       <c r="D43" s="5"/>
     </row>
     <row r="44" spans="2:4">
       <c r="B44" s="5" t="s">
-        <v>933</v>
+        <v>961</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>934</v>
+        <v>962</v>
       </c>
       <c r="D44" s="5"/>
     </row>
@@ -8565,7 +8999,7 @@
         <v>185</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>935</v>
+        <v>963</v>
       </c>
       <c r="D45" s="5"/>
     </row>
@@ -8574,7 +9008,7 @@
         <v>190</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>936</v>
+        <v>964</v>
       </c>
       <c r="D46" s="5"/>
     </row>
@@ -8583,27 +9017,27 @@
         <v>195</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>937</v>
+        <v>965</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>938</v>
+        <v>966</v>
       </c>
     </row>
     <row r="48" spans="2:4">
       <c r="B48" s="5" t="s">
-        <v>939</v>
+        <v>967</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>940</v>
+        <v>968</v>
       </c>
       <c r="D48" s="5"/>
     </row>
     <row r="49" spans="2:4">
       <c r="B49" s="5" t="s">
-        <v>941</v>
+        <v>969</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>942</v>
+        <v>970</v>
       </c>
       <c r="D49" s="5"/>
     </row>
@@ -8612,7 +9046,7 @@
         <v>208</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>943</v>
+        <v>971</v>
       </c>
       <c r="D50" s="5"/>
     </row>
@@ -8621,7 +9055,7 @@
         <v>213</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>944</v>
+        <v>972</v>
       </c>
       <c r="D51" s="5"/>
     </row>
@@ -8630,25 +9064,25 @@
         <v>218</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>945</v>
+        <v>973</v>
       </c>
       <c r="D52" s="5"/>
     </row>
     <row r="53" spans="2:4">
       <c r="B53" s="5" t="s">
-        <v>946</v>
+        <v>974</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>947</v>
+        <v>975</v>
       </c>
       <c r="D53" s="5"/>
     </row>
     <row r="54" spans="2:4">
       <c r="B54" s="5" t="s">
-        <v>948</v>
+        <v>976</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>949</v>
+        <v>977</v>
       </c>
       <c r="D54" s="5"/>
     </row>
@@ -8657,7 +9091,7 @@
         <v>231</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>950</v>
+        <v>978</v>
       </c>
       <c r="D55" s="5"/>
     </row>
@@ -8666,7 +9100,7 @@
         <v>236</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>951</v>
+        <v>979</v>
       </c>
       <c r="D56" s="5"/>
     </row>
@@ -8675,27 +9109,27 @@
         <v>58</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>952</v>
+        <v>980</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>953</v>
+        <v>981</v>
       </c>
     </row>
     <row r="58" spans="2:4">
       <c r="B58" s="5" t="s">
-        <v>954</v>
+        <v>982</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>955</v>
+        <v>983</v>
       </c>
       <c r="D58" s="5"/>
     </row>
     <row r="59" spans="2:4">
       <c r="B59" s="5" t="s">
-        <v>956</v>
+        <v>984</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>957</v>
+        <v>985</v>
       </c>
       <c r="D59" s="5"/>
     </row>
@@ -8704,7 +9138,7 @@
         <v>253</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>958</v>
+        <v>986</v>
       </c>
       <c r="D60" s="5"/>
     </row>
@@ -8713,7 +9147,7 @@
         <v>258</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>959</v>
+        <v>987</v>
       </c>
       <c r="D61" s="5"/>
     </row>
@@ -8722,25 +9156,25 @@
         <v>263</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>960</v>
+        <v>988</v>
       </c>
       <c r="D62" s="5"/>
     </row>
     <row r="63" spans="2:4">
       <c r="B63" s="5" t="s">
-        <v>961</v>
+        <v>989</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>962</v>
+        <v>990</v>
       </c>
       <c r="D63" s="5"/>
     </row>
     <row r="64" spans="2:4">
       <c r="B64" s="5" t="s">
-        <v>963</v>
+        <v>991</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>964</v>
+        <v>992</v>
       </c>
       <c r="D64" s="5"/>
     </row>
@@ -8749,7 +9183,7 @@
         <v>276</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>965</v>
+        <v>993</v>
       </c>
       <c r="D65" s="5"/>
     </row>
@@ -8758,7 +9192,7 @@
         <v>281</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>966</v>
+        <v>994</v>
       </c>
       <c r="D66" s="5"/>
     </row>
@@ -8767,27 +9201,27 @@
         <v>286</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>967</v>
+        <v>995</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>968</v>
+        <v>996</v>
       </c>
     </row>
     <row r="68" spans="2:4">
       <c r="B68" s="5" t="s">
-        <v>969</v>
+        <v>997</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>970</v>
+        <v>998</v>
       </c>
       <c r="D68" s="5"/>
     </row>
     <row r="69" spans="2:4">
       <c r="B69" s="5" t="s">
-        <v>971</v>
+        <v>999</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>972</v>
+        <v>1000</v>
       </c>
       <c r="D69" s="5"/>
     </row>
@@ -8796,7 +9230,7 @@
         <v>299</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>973</v>
+        <v>1001</v>
       </c>
       <c r="D70" s="5"/>
     </row>
@@ -8805,7 +9239,7 @@
         <v>304</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>974</v>
+        <v>1002</v>
       </c>
       <c r="D71" s="5"/>
     </row>
@@ -8814,25 +9248,25 @@
         <v>309</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>975</v>
+        <v>1003</v>
       </c>
       <c r="D72" s="5"/>
     </row>
     <row r="73" spans="2:4">
       <c r="B73" s="5" t="s">
-        <v>976</v>
+        <v>1004</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>977</v>
+        <v>1005</v>
       </c>
       <c r="D73" s="5"/>
     </row>
     <row r="74" spans="2:4">
       <c r="B74" s="5" t="s">
-        <v>978</v>
+        <v>1006</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>979</v>
+        <v>1007</v>
       </c>
       <c r="D74" s="5"/>
     </row>
@@ -8841,7 +9275,7 @@
         <v>322</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="D75" s="5"/>
     </row>
@@ -8850,7 +9284,7 @@
         <v>327</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>981</v>
+        <v>1009</v>
       </c>
       <c r="D76" s="5"/>
     </row>
@@ -8859,27 +9293,27 @@
         <v>332</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>982</v>
+        <v>1010</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>983</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="78" spans="2:4">
       <c r="B78" s="5" t="s">
-        <v>984</v>
+        <v>1012</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>985</v>
+        <v>1013</v>
       </c>
       <c r="D78" s="5"/>
     </row>
     <row r="79" spans="2:4">
       <c r="B79" s="5" t="s">
-        <v>986</v>
+        <v>1014</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>987</v>
+        <v>1015</v>
       </c>
       <c r="D79" s="5"/>
     </row>
@@ -8888,7 +9322,7 @@
         <v>345</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>988</v>
+        <v>1016</v>
       </c>
       <c r="D80" s="5"/>
     </row>
@@ -8897,7 +9331,7 @@
         <v>350</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>989</v>
+        <v>1017</v>
       </c>
       <c r="D81" s="5"/>
     </row>
@@ -8906,25 +9340,25 @@
         <v>355</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>990</v>
+        <v>1018</v>
       </c>
       <c r="D82" s="5"/>
     </row>
     <row r="83" spans="2:4">
       <c r="B83" s="5" t="s">
-        <v>991</v>
+        <v>1019</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>992</v>
+        <v>1020</v>
       </c>
       <c r="D83" s="5"/>
     </row>
     <row r="84" spans="2:4">
       <c r="B84" s="5" t="s">
-        <v>993</v>
+        <v>1021</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>994</v>
+        <v>1022</v>
       </c>
       <c r="D84" s="5"/>
     </row>
@@ -8933,7 +9367,7 @@
         <v>368</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>995</v>
+        <v>1023</v>
       </c>
       <c r="D85" s="5"/>
     </row>
@@ -8942,7 +9376,7 @@
         <v>373</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>996</v>
+        <v>1024</v>
       </c>
       <c r="D86" s="5"/>
     </row>
@@ -8951,27 +9385,27 @@
         <v>378</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>997</v>
+        <v>1025</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>998</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="88" spans="2:4">
       <c r="B88" s="5" t="s">
-        <v>999</v>
+        <v>1027</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>1000</v>
+        <v>1028</v>
       </c>
       <c r="D88" s="5"/>
     </row>
     <row r="89" spans="2:4">
       <c r="B89" s="5" t="s">
-        <v>1001</v>
+        <v>1029</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>1002</v>
+        <v>1030</v>
       </c>
       <c r="D89" s="5"/>
     </row>
@@ -8980,7 +9414,7 @@
         <v>391</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>1003</v>
+        <v>1031</v>
       </c>
       <c r="D90" s="5"/>
     </row>
@@ -8989,7 +9423,7 @@
         <v>396</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>1004</v>
+        <v>1032</v>
       </c>
       <c r="D91" s="5"/>
     </row>
@@ -8998,25 +9432,25 @@
         <v>401</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>1005</v>
+        <v>1033</v>
       </c>
       <c r="D92" s="5"/>
     </row>
     <row r="93" spans="2:4">
       <c r="B93" s="5" t="s">
-        <v>1006</v>
+        <v>1034</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>1007</v>
+        <v>1035</v>
       </c>
       <c r="D93" s="5"/>
     </row>
     <row r="94" spans="2:4">
       <c r="B94" s="5" t="s">
-        <v>1008</v>
+        <v>1036</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>1009</v>
+        <v>1037</v>
       </c>
       <c r="D94" s="5"/>
     </row>
@@ -9025,7 +9459,7 @@
         <v>414</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>1010</v>
+        <v>1038</v>
       </c>
       <c r="D95" s="5"/>
     </row>
@@ -9034,7 +9468,7 @@
         <v>419</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>1011</v>
+        <v>1039</v>
       </c>
       <c r="D96" s="5"/>
     </row>
@@ -9043,27 +9477,27 @@
         <v>424</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>1012</v>
+        <v>1040</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>1013</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="98" spans="2:4">
       <c r="B98" s="5" t="s">
-        <v>1014</v>
+        <v>1042</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>1015</v>
+        <v>1043</v>
       </c>
       <c r="D98" s="5"/>
     </row>
     <row r="99" spans="2:4">
       <c r="B99" s="5" t="s">
-        <v>1016</v>
+        <v>1044</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>1017</v>
+        <v>1045</v>
       </c>
       <c r="D99" s="5"/>
     </row>
@@ -9072,7 +9506,7 @@
         <v>437</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>1018</v>
+        <v>1046</v>
       </c>
       <c r="D100" s="5"/>
     </row>
@@ -9081,7 +9515,7 @@
         <v>442</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>1019</v>
+        <v>1047</v>
       </c>
       <c r="D101" s="5"/>
     </row>
@@ -9090,25 +9524,25 @@
         <v>447</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>1020</v>
+        <v>1048</v>
       </c>
       <c r="D102" s="5"/>
     </row>
     <row r="103" spans="2:4">
       <c r="B103" s="5" t="s">
-        <v>1021</v>
+        <v>1049</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>1022</v>
+        <v>1050</v>
       </c>
       <c r="D103" s="5"/>
     </row>
     <row r="104" spans="2:4">
       <c r="B104" s="5" t="s">
-        <v>1023</v>
+        <v>1051</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>1024</v>
+        <v>1052</v>
       </c>
       <c r="D104" s="5"/>
     </row>
@@ -9117,7 +9551,7 @@
         <v>460</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>1025</v>
+        <v>1053</v>
       </c>
       <c r="D105" s="5"/>
     </row>
@@ -9126,19 +9560,19 @@
         <v>465</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>1026</v>
+        <v>1054</v>
       </c>
       <c r="D106" s="5"/>
     </row>
     <row r="107" spans="2:4">
       <c r="B107" s="5" t="s">
-        <v>883</v>
+        <v>911</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>1027</v>
+        <v>1055</v>
       </c>
       <c r="D107" s="5" t="s">
-        <v>1028</v>
+        <v>1056</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(i18n)!: split localization catalog from config tables
Add first-class localization schema, text keys, independent LocaleCatalog loading, and i18n binary/json exports. Regenerate showcase outputs without Localization as a normal business table.
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Core.xlsx
+++ b/examples/showcase/data/Core.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Item" sheetId="1" r:id="rId1"/>
-    <sheet name="GameSettings" sheetId="2" r:id="rId2"/>
-    <sheet name="MaintenanceWindow" sheetId="3" r:id="rId3"/>
-    <sheet name="Localization" sheetId="4" r:id="rId4"/>
-    <sheet name="LevelExp" sheetId="5" r:id="rId5"/>
+    <sheet name="LevelExp" sheetId="2" r:id="rId2"/>
+    <sheet name="GameSettings" sheetId="3" r:id="rId3"/>
+    <sheet name="MaintenanceWindow" sheetId="4" r:id="rId4"/>
+    <sheet name="Localization" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -515,8 +515,47 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+    <author>Sora</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Localization key
+Field: key
+Type: string
+Scope: all
+Key: yes</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1789" uniqueCount="972">
   <si>
     <t>@table</t>
   </si>
@@ -2174,6 +2213,372 @@
     <t>tier,2|power,131</t>
   </si>
   <si>
+    <t>LevelExp</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>96c986fb1afe3d5a</t>
+  </si>
+  <si>
+    <t>exp</t>
+  </si>
+  <si>
+    <t>unlock_feature</t>
+  </si>
+  <si>
+    <t>i64</t>
+  </si>
+  <si>
+    <t>optional&lt;string&gt;</t>
+  </si>
+  <si>
+    <t>key;range=1..100</t>
+  </si>
+  <si>
+    <t>range=0..999999999</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>900</t>
+  </si>
+  <si>
+    <t>1600</t>
+  </si>
+  <si>
+    <t>2500</t>
+  </si>
+  <si>
+    <t>3600</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>4900</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>6400</t>
+  </si>
+  <si>
+    <t>8100</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>feature_10</t>
+  </si>
+  <si>
+    <t>12100</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>14400</t>
+  </si>
+  <si>
+    <t>16900</t>
+  </si>
+  <si>
+    <t>19600</t>
+  </si>
+  <si>
+    <t>22500</t>
+  </si>
+  <si>
+    <t>25600</t>
+  </si>
+  <si>
+    <t>28900</t>
+  </si>
+  <si>
+    <t>32400</t>
+  </si>
+  <si>
+    <t>36100</t>
+  </si>
+  <si>
+    <t>40000</t>
+  </si>
+  <si>
+    <t>feature_20</t>
+  </si>
+  <si>
+    <t>44100</t>
+  </si>
+  <si>
+    <t>48400</t>
+  </si>
+  <si>
+    <t>52900</t>
+  </si>
+  <si>
+    <t>57600</t>
+  </si>
+  <si>
+    <t>62500</t>
+  </si>
+  <si>
+    <t>67600</t>
+  </si>
+  <si>
+    <t>72900</t>
+  </si>
+  <si>
+    <t>78400</t>
+  </si>
+  <si>
+    <t>84100</t>
+  </si>
+  <si>
+    <t>90000</t>
+  </si>
+  <si>
+    <t>feature_30</t>
+  </si>
+  <si>
+    <t>96100</t>
+  </si>
+  <si>
+    <t>102400</t>
+  </si>
+  <si>
+    <t>108900</t>
+  </si>
+  <si>
+    <t>115600</t>
+  </si>
+  <si>
+    <t>122500</t>
+  </si>
+  <si>
+    <t>129600</t>
+  </si>
+  <si>
+    <t>136900</t>
+  </si>
+  <si>
+    <t>144400</t>
+  </si>
+  <si>
+    <t>152100</t>
+  </si>
+  <si>
+    <t>160000</t>
+  </si>
+  <si>
+    <t>feature_40</t>
+  </si>
+  <si>
+    <t>168100</t>
+  </si>
+  <si>
+    <t>176400</t>
+  </si>
+  <si>
+    <t>184900</t>
+  </si>
+  <si>
+    <t>193600</t>
+  </si>
+  <si>
+    <t>202500</t>
+  </si>
+  <si>
+    <t>211600</t>
+  </si>
+  <si>
+    <t>220900</t>
+  </si>
+  <si>
+    <t>230400</t>
+  </si>
+  <si>
+    <t>240100</t>
+  </si>
+  <si>
+    <t>250000</t>
+  </si>
+  <si>
+    <t>feature_50</t>
+  </si>
+  <si>
+    <t>260100</t>
+  </si>
+  <si>
+    <t>270400</t>
+  </si>
+  <si>
+    <t>280900</t>
+  </si>
+  <si>
+    <t>291600</t>
+  </si>
+  <si>
+    <t>302500</t>
+  </si>
+  <si>
+    <t>313600</t>
+  </si>
+  <si>
+    <t>324900</t>
+  </si>
+  <si>
+    <t>336400</t>
+  </si>
+  <si>
+    <t>348100</t>
+  </si>
+  <si>
+    <t>360000</t>
+  </si>
+  <si>
+    <t>feature_60</t>
+  </si>
+  <si>
+    <t>372100</t>
+  </si>
+  <si>
+    <t>384400</t>
+  </si>
+  <si>
+    <t>396900</t>
+  </si>
+  <si>
+    <t>409600</t>
+  </si>
+  <si>
+    <t>422500</t>
+  </si>
+  <si>
+    <t>435600</t>
+  </si>
+  <si>
+    <t>448900</t>
+  </si>
+  <si>
+    <t>462400</t>
+  </si>
+  <si>
+    <t>476100</t>
+  </si>
+  <si>
+    <t>490000</t>
+  </si>
+  <si>
+    <t>feature_70</t>
+  </si>
+  <si>
+    <t>504100</t>
+  </si>
+  <si>
+    <t>518400</t>
+  </si>
+  <si>
+    <t>532900</t>
+  </si>
+  <si>
+    <t>547600</t>
+  </si>
+  <si>
+    <t>562500</t>
+  </si>
+  <si>
+    <t>577600</t>
+  </si>
+  <si>
+    <t>592900</t>
+  </si>
+  <si>
+    <t>608400</t>
+  </si>
+  <si>
+    <t>624100</t>
+  </si>
+  <si>
+    <t>640000</t>
+  </si>
+  <si>
+    <t>feature_80</t>
+  </si>
+  <si>
+    <t>656100</t>
+  </si>
+  <si>
+    <t>672400</t>
+  </si>
+  <si>
+    <t>688900</t>
+  </si>
+  <si>
+    <t>705600</t>
+  </si>
+  <si>
+    <t>722500</t>
+  </si>
+  <si>
+    <t>739600</t>
+  </si>
+  <si>
+    <t>756900</t>
+  </si>
+  <si>
+    <t>774400</t>
+  </si>
+  <si>
+    <t>792100</t>
+  </si>
+  <si>
+    <t>810000</t>
+  </si>
+  <si>
+    <t>feature_90</t>
+  </si>
+  <si>
+    <t>828100</t>
+  </si>
+  <si>
+    <t>846400</t>
+  </si>
+  <si>
+    <t>864900</t>
+  </si>
+  <si>
+    <t>883600</t>
+  </si>
+  <si>
+    <t>902500</t>
+  </si>
+  <si>
+    <t>921600</t>
+  </si>
+  <si>
+    <t>940900</t>
+  </si>
+  <si>
+    <t>960400</t>
+  </si>
+  <si>
+    <t>980100</t>
+  </si>
+  <si>
+    <t>1000000</t>
+  </si>
+  <si>
+    <t>feature_100</t>
+  </si>
+  <si>
     <t>GameSettings</t>
   </si>
   <si>
@@ -2297,9 +2702,6 @@
     <t>reason</t>
   </si>
   <si>
-    <t>optional&lt;string&gt;</t>
-  </si>
-  <si>
     <t>range=1..1440</t>
   </si>
   <si>
@@ -2312,7 +2714,7 @@
     <t>Localization</t>
   </si>
   <si>
-    <t>7725a2f29e13764d</t>
+    <t>56eb26c49c6d18a3</t>
   </si>
   <si>
     <t>zh_cn</t>
@@ -2324,7 +2726,7 @@
     <t>note</t>
   </si>
   <si>
-    <t>key;length=3..64</t>
+    <t>Localization key</t>
   </si>
   <si>
     <t>loc_001</t>
@@ -3069,369 +3471,6 @@
   </si>
   <si>
     <t>note 80</t>
-  </si>
-  <si>
-    <t>LevelExp</t>
-  </si>
-  <si>
-    <t>level</t>
-  </si>
-  <si>
-    <t>96c986fb1afe3d5a</t>
-  </si>
-  <si>
-    <t>exp</t>
-  </si>
-  <si>
-    <t>unlock_feature</t>
-  </si>
-  <si>
-    <t>i64</t>
-  </si>
-  <si>
-    <t>key;range=1..100</t>
-  </si>
-  <si>
-    <t>range=0..999999999</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>400</t>
-  </si>
-  <si>
-    <t>900</t>
-  </si>
-  <si>
-    <t>1600</t>
-  </si>
-  <si>
-    <t>2500</t>
-  </si>
-  <si>
-    <t>3600</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>4900</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>6400</t>
-  </si>
-  <si>
-    <t>8100</t>
-  </si>
-  <si>
-    <t>10000</t>
-  </si>
-  <si>
-    <t>feature_10</t>
-  </si>
-  <si>
-    <t>12100</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>14400</t>
-  </si>
-  <si>
-    <t>16900</t>
-  </si>
-  <si>
-    <t>19600</t>
-  </si>
-  <si>
-    <t>22500</t>
-  </si>
-  <si>
-    <t>25600</t>
-  </si>
-  <si>
-    <t>28900</t>
-  </si>
-  <si>
-    <t>32400</t>
-  </si>
-  <si>
-    <t>36100</t>
-  </si>
-  <si>
-    <t>40000</t>
-  </si>
-  <si>
-    <t>feature_20</t>
-  </si>
-  <si>
-    <t>44100</t>
-  </si>
-  <si>
-    <t>48400</t>
-  </si>
-  <si>
-    <t>52900</t>
-  </si>
-  <si>
-    <t>57600</t>
-  </si>
-  <si>
-    <t>62500</t>
-  </si>
-  <si>
-    <t>67600</t>
-  </si>
-  <si>
-    <t>72900</t>
-  </si>
-  <si>
-    <t>78400</t>
-  </si>
-  <si>
-    <t>84100</t>
-  </si>
-  <si>
-    <t>90000</t>
-  </si>
-  <si>
-    <t>feature_30</t>
-  </si>
-  <si>
-    <t>96100</t>
-  </si>
-  <si>
-    <t>102400</t>
-  </si>
-  <si>
-    <t>108900</t>
-  </si>
-  <si>
-    <t>115600</t>
-  </si>
-  <si>
-    <t>122500</t>
-  </si>
-  <si>
-    <t>129600</t>
-  </si>
-  <si>
-    <t>136900</t>
-  </si>
-  <si>
-    <t>144400</t>
-  </si>
-  <si>
-    <t>152100</t>
-  </si>
-  <si>
-    <t>160000</t>
-  </si>
-  <si>
-    <t>feature_40</t>
-  </si>
-  <si>
-    <t>168100</t>
-  </si>
-  <si>
-    <t>176400</t>
-  </si>
-  <si>
-    <t>184900</t>
-  </si>
-  <si>
-    <t>193600</t>
-  </si>
-  <si>
-    <t>202500</t>
-  </si>
-  <si>
-    <t>211600</t>
-  </si>
-  <si>
-    <t>220900</t>
-  </si>
-  <si>
-    <t>230400</t>
-  </si>
-  <si>
-    <t>240100</t>
-  </si>
-  <si>
-    <t>250000</t>
-  </si>
-  <si>
-    <t>feature_50</t>
-  </si>
-  <si>
-    <t>260100</t>
-  </si>
-  <si>
-    <t>270400</t>
-  </si>
-  <si>
-    <t>280900</t>
-  </si>
-  <si>
-    <t>291600</t>
-  </si>
-  <si>
-    <t>302500</t>
-  </si>
-  <si>
-    <t>313600</t>
-  </si>
-  <si>
-    <t>324900</t>
-  </si>
-  <si>
-    <t>336400</t>
-  </si>
-  <si>
-    <t>348100</t>
-  </si>
-  <si>
-    <t>360000</t>
-  </si>
-  <si>
-    <t>feature_60</t>
-  </si>
-  <si>
-    <t>372100</t>
-  </si>
-  <si>
-    <t>384400</t>
-  </si>
-  <si>
-    <t>396900</t>
-  </si>
-  <si>
-    <t>409600</t>
-  </si>
-  <si>
-    <t>422500</t>
-  </si>
-  <si>
-    <t>435600</t>
-  </si>
-  <si>
-    <t>448900</t>
-  </si>
-  <si>
-    <t>462400</t>
-  </si>
-  <si>
-    <t>476100</t>
-  </si>
-  <si>
-    <t>490000</t>
-  </si>
-  <si>
-    <t>feature_70</t>
-  </si>
-  <si>
-    <t>504100</t>
-  </si>
-  <si>
-    <t>518400</t>
-  </si>
-  <si>
-    <t>532900</t>
-  </si>
-  <si>
-    <t>547600</t>
-  </si>
-  <si>
-    <t>562500</t>
-  </si>
-  <si>
-    <t>577600</t>
-  </si>
-  <si>
-    <t>592900</t>
-  </si>
-  <si>
-    <t>608400</t>
-  </si>
-  <si>
-    <t>624100</t>
-  </si>
-  <si>
-    <t>640000</t>
-  </si>
-  <si>
-    <t>feature_80</t>
-  </si>
-  <si>
-    <t>656100</t>
-  </si>
-  <si>
-    <t>672400</t>
-  </si>
-  <si>
-    <t>688900</t>
-  </si>
-  <si>
-    <t>705600</t>
-  </si>
-  <si>
-    <t>722500</t>
-  </si>
-  <si>
-    <t>739600</t>
-  </si>
-  <si>
-    <t>756900</t>
-  </si>
-  <si>
-    <t>774400</t>
-  </si>
-  <si>
-    <t>792100</t>
-  </si>
-  <si>
-    <t>810000</t>
-  </si>
-  <si>
-    <t>feature_90</t>
-  </si>
-  <si>
-    <t>828100</t>
-  </si>
-  <si>
-    <t>846400</t>
-  </si>
-  <si>
-    <t>864900</t>
-  </si>
-  <si>
-    <t>883600</t>
-  </si>
-  <si>
-    <t>902500</t>
-  </si>
-  <si>
-    <t>921600</t>
-  </si>
-  <si>
-    <t>940900</t>
-  </si>
-  <si>
-    <t>960400</t>
-  </si>
-  <si>
-    <t>980100</t>
-  </si>
-  <si>
-    <t>1000000</t>
-  </si>
-  <si>
-    <t>feature_100</t>
   </si>
 </sst>
 </file>
@@ -3485,7 +3524,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3540,6 +3579,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F4F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAFAFA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -3568,7 +3619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3598,6 +3649,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -7679,6 +7736,1059 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J107"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="6" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" style="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="B8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="B10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="B11" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="B12" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="B13" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="D13" s="6"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="B14" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="D18" s="6"/>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="B19" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="D19" s="6"/>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="B20" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="D20" s="6"/>
+    </row>
+    <row r="21" spans="2:4">
+      <c r="B21" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D21" s="6"/>
+    </row>
+    <row r="22" spans="2:4">
+      <c r="B22" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="D22" s="6"/>
+    </row>
+    <row r="23" spans="2:4">
+      <c r="B23" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="D23" s="6"/>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="B24" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="D24" s="6"/>
+    </row>
+    <row r="25" spans="2:4">
+      <c r="B25" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="D25" s="6"/>
+    </row>
+    <row r="26" spans="2:4">
+      <c r="B26" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="D26" s="6"/>
+    </row>
+    <row r="27" spans="2:4">
+      <c r="B27" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4">
+      <c r="B28" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="D28" s="6"/>
+    </row>
+    <row r="29" spans="2:4">
+      <c r="B29" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="D29" s="6"/>
+    </row>
+    <row r="30" spans="2:4">
+      <c r="B30" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="D30" s="6"/>
+    </row>
+    <row r="31" spans="2:4">
+      <c r="B31" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="D31" s="6"/>
+    </row>
+    <row r="32" spans="2:4">
+      <c r="B32" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="D32" s="6"/>
+    </row>
+    <row r="33" spans="2:4">
+      <c r="B33" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" spans="2:4">
+      <c r="B34" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="D34" s="6"/>
+    </row>
+    <row r="35" spans="2:4">
+      <c r="B35" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="D35" s="6"/>
+    </row>
+    <row r="36" spans="2:4">
+      <c r="B36" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="D36" s="6"/>
+    </row>
+    <row r="37" spans="2:4">
+      <c r="B37" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4">
+      <c r="B38" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>597</v>
+      </c>
+      <c r="D38" s="6"/>
+    </row>
+    <row r="39" spans="2:4">
+      <c r="B39" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="D39" s="6"/>
+    </row>
+    <row r="40" spans="2:4">
+      <c r="B40" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="D40" s="6"/>
+    </row>
+    <row r="41" spans="2:4">
+      <c r="B41" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="D41" s="6"/>
+    </row>
+    <row r="42" spans="2:4">
+      <c r="B42" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="D42" s="6"/>
+    </row>
+    <row r="43" spans="2:4">
+      <c r="B43" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="D43" s="6"/>
+    </row>
+    <row r="44" spans="2:4">
+      <c r="B44" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="D44" s="6"/>
+    </row>
+    <row r="45" spans="2:4">
+      <c r="B45" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="D45" s="6"/>
+    </row>
+    <row r="46" spans="2:4">
+      <c r="B46" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="D46" s="6"/>
+    </row>
+    <row r="47" spans="2:4">
+      <c r="B47" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="48" spans="2:4">
+      <c r="B48" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="D48" s="6"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>609</v>
+      </c>
+      <c r="D49" s="6"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="D50" s="6"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="D51" s="6"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="D52" s="6"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="D53" s="6"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="D54" s="6"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="D55" s="6"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="D56" s="6"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>619</v>
+      </c>
+      <c r="D58" s="6"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="D59" s="6"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="D60" s="6"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="D61" s="6"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="D62" s="6"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="D63" s="6"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="D64" s="6"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="D65" s="6"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="D66" s="6"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="D68" s="6"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="D69" s="6"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="D70" s="6"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="D71" s="6"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="D72" s="6"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="D73" s="6"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="D74" s="6"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="D75" s="6"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="D76" s="6"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="D78" s="6"/>
+    </row>
+    <row r="79" spans="2:4">
+      <c r="B79" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="D79" s="6"/>
+    </row>
+    <row r="80" spans="2:4">
+      <c r="B80" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="D80" s="6"/>
+    </row>
+    <row r="81" spans="2:4">
+      <c r="B81" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="D81" s="6"/>
+    </row>
+    <row r="82" spans="2:4">
+      <c r="B82" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="D82" s="6"/>
+    </row>
+    <row r="83" spans="2:4">
+      <c r="B83" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="D83" s="6"/>
+    </row>
+    <row r="84" spans="2:4">
+      <c r="B84" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="D84" s="6"/>
+    </row>
+    <row r="85" spans="2:4">
+      <c r="B85" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="D85" s="6"/>
+    </row>
+    <row r="86" spans="2:4">
+      <c r="B86" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="D86" s="6"/>
+    </row>
+    <row r="87" spans="2:4">
+      <c r="B87" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="88" spans="2:4">
+      <c r="B88" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="D88" s="6"/>
+    </row>
+    <row r="89" spans="2:4">
+      <c r="B89" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="D89" s="6"/>
+    </row>
+    <row r="90" spans="2:4">
+      <c r="B90" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="D90" s="6"/>
+    </row>
+    <row r="91" spans="2:4">
+      <c r="B91" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="D91" s="6"/>
+    </row>
+    <row r="92" spans="2:4">
+      <c r="B92" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="D92" s="6"/>
+    </row>
+    <row r="93" spans="2:4">
+      <c r="B93" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="D93" s="6"/>
+    </row>
+    <row r="94" spans="2:4">
+      <c r="B94" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="D94" s="6"/>
+    </row>
+    <row r="95" spans="2:4">
+      <c r="B95" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="D95" s="6"/>
+    </row>
+    <row r="96" spans="2:4">
+      <c r="B96" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="D96" s="6"/>
+    </row>
+    <row r="97" spans="2:4">
+      <c r="B97" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="98" spans="2:4">
+      <c r="B98" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="D98" s="6"/>
+    </row>
+    <row r="99" spans="2:4">
+      <c r="B99" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="D99" s="6"/>
+    </row>
+    <row r="100" spans="2:4">
+      <c r="B100" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="D100" s="6"/>
+    </row>
+    <row r="101" spans="2:4">
+      <c r="B101" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="D101" s="6"/>
+    </row>
+    <row r="102" spans="2:4">
+      <c r="B102" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="D102" s="6"/>
+    </row>
+    <row r="103" spans="2:4">
+      <c r="B103" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="D103" s="6"/>
+    </row>
+    <row r="104" spans="2:4">
+      <c r="B104" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="D104" s="6"/>
+    </row>
+    <row r="105" spans="2:4">
+      <c r="B105" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="D105" s="6"/>
+    </row>
+    <row r="106" spans="2:4">
+      <c r="B106" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="D106" s="6"/>
+    </row>
+    <row r="107" spans="2:4">
+      <c r="B107" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>673</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 100." promptTitle="Integer range" prompt="Enter an integer from 1 to 100." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 999999999." promptTitle="Integer range" prompt="Enter an integer from 0 to 999999999." sqref="C8:C1007">
+      <formula1>0</formula1>
+      <formula2>999999999</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -7698,13 +8808,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>552</v>
+        <v>674</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>553</v>
+        <v>675</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -7720,7 +8830,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>554</v>
+        <v>676</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7728,31 +8838,31 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>555</v>
+        <v>677</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>556</v>
+        <v>678</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>557</v>
+        <v>679</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>558</v>
+        <v>680</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>559</v>
+        <v>681</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>560</v>
+        <v>682</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>561</v>
+        <v>683</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>562</v>
+        <v>684</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>563</v>
+        <v>685</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -7760,31 +8870,31 @@
         <v>19</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>555</v>
+        <v>677</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>556</v>
+        <v>678</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>557</v>
+        <v>679</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>558</v>
+        <v>680</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>559</v>
+        <v>681</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>560</v>
+        <v>682</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>561</v>
+        <v>683</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>562</v>
+        <v>684</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>563</v>
+        <v>685</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -7801,22 +8911,22 @@
         <v>21</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>564</v>
+        <v>686</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>565</v>
+        <v>687</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>566</v>
+        <v>688</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>567</v>
+        <v>689</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>568</v>
+        <v>690</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>569</v>
+        <v>691</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -7857,26 +8967,26 @@
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
-        <v>570</v>
+        <v>692</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>571</v>
+        <v>693</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>572</v>
+        <v>694</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>573</v>
+        <v>695</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6" t="s">
-        <v>574</v>
+        <v>696</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>575</v>
+        <v>697</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>576</v>
+        <v>698</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
@@ -7889,43 +8999,43 @@
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8" t="s">
-        <v>577</v>
+        <v>699</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>578</v>
+        <v>700</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>579</v>
+        <v>701</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>580</v>
+        <v>702</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="6" t="s">
-        <v>581</v>
+        <v>703</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>438</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
-        <v>582</v>
+        <v>704</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>584</v>
+        <v>706</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>585</v>
+        <v>707</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>586</v>
+        <v>708</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>576</v>
+        <v>698</v>
       </c>
     </row>
   </sheetData>
@@ -7944,7 +9054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7959,13 +9069,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>587</v>
+        <v>709</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>588</v>
+        <v>710</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -7981,7 +9091,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>589</v>
+        <v>711</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -7989,16 +9099,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>555</v>
+        <v>677</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>590</v>
+        <v>712</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>591</v>
+        <v>713</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>592</v>
+        <v>714</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -8006,16 +9116,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>555</v>
+        <v>677</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>590</v>
+        <v>712</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>591</v>
+        <v>713</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>592</v>
+        <v>714</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -8032,7 +9142,7 @@
         <v>21</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>593</v>
+        <v>558</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -8059,7 +9169,7 @@
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
-        <v>594</v>
+        <v>715</v>
       </c>
       <c r="E6" s="6"/>
     </row>
@@ -8074,16 +9184,16 @@
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="6" t="s">
-        <v>581</v>
+        <v>703</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>595</v>
+        <v>716</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>382</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>596</v>
+        <v>717</v>
       </c>
     </row>
   </sheetData>
@@ -8097,14 +9207,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="4" width="12.7109375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="6" customWidth="1"/>
+    <col min="3" max="4" width="12.7109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -8112,7 +9223,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>597</v>
+        <v>718</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8120,7 +9231,7 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
@@ -8136,7 +9247,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>598</v>
+        <v>719</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -8147,13 +9258,13 @@
         <v>29</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>599</v>
+        <v>720</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>600</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>601</v>
+        <v>721</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>722</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -8164,13 +9275,13 @@
         <v>29</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>599</v>
+        <v>720</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>600</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>601</v>
+        <v>721</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>722</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -8186,8 +9297,8 @@
       <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>593</v>
+      <c r="E4" s="11" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -8203,7 +9314,7 @@
       <c r="D5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -8212,2051 +9323,929 @@
         <v>28</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>602</v>
+        <v>29</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="8"/>
+      <c r="B7" s="8" t="s">
+        <v>723</v>
+      </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="6" t="s">
-        <v>603</v>
+        <v>724</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>604</v>
+        <v>725</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>605</v>
-      </c>
-      <c r="E8" s="6"/>
+        <v>726</v>
+      </c>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="6" t="s">
-        <v>606</v>
+        <v>727</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>607</v>
+        <v>728</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>608</v>
-      </c>
-      <c r="E9" s="6"/>
+        <v>729</v>
+      </c>
     </row>
     <row r="10" spans="1:10">
       <c r="B10" s="6" t="s">
-        <v>609</v>
+        <v>730</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>610</v>
+        <v>731</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>611</v>
-      </c>
-      <c r="E10" s="6"/>
+        <v>732</v>
+      </c>
     </row>
     <row r="11" spans="1:10">
       <c r="B11" s="6" t="s">
-        <v>612</v>
+        <v>733</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>613</v>
+        <v>734</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>614</v>
-      </c>
-      <c r="E11" s="6"/>
+        <v>735</v>
+      </c>
     </row>
     <row r="12" spans="1:10">
       <c r="B12" s="6" t="s">
-        <v>615</v>
+        <v>736</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>616</v>
+        <v>737</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>617</v>
-      </c>
-      <c r="E12" s="6"/>
+        <v>738</v>
+      </c>
     </row>
     <row r="13" spans="1:10">
       <c r="B13" s="6" t="s">
-        <v>618</v>
+        <v>739</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>619</v>
+        <v>740</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>620</v>
-      </c>
-      <c r="E13" s="6"/>
+        <v>741</v>
+      </c>
     </row>
     <row r="14" spans="1:10">
       <c r="B14" s="6" t="s">
-        <v>621</v>
+        <v>742</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>622</v>
+        <v>743</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>623</v>
-      </c>
-      <c r="E14" s="6"/>
+        <v>744</v>
+      </c>
     </row>
     <row r="15" spans="1:10">
       <c r="B15" s="6" t="s">
-        <v>624</v>
+        <v>745</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>625</v>
+        <v>746</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>626</v>
-      </c>
-      <c r="E15" s="6"/>
+        <v>747</v>
+      </c>
     </row>
     <row r="16" spans="1:10">
       <c r="B16" s="6" t="s">
-        <v>627</v>
+        <v>748</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>628</v>
+        <v>749</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>629</v>
-      </c>
-      <c r="E16" s="6"/>
+        <v>750</v>
+      </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="6" t="s">
-        <v>630</v>
+        <v>751</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>631</v>
+        <v>752</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>632</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>633</v>
+        <v>753</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>754</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="6" t="s">
-        <v>634</v>
+        <v>755</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>635</v>
+        <v>756</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>636</v>
-      </c>
-      <c r="E18" s="6"/>
+        <v>757</v>
+      </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="6" t="s">
-        <v>637</v>
+        <v>758</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>638</v>
+        <v>759</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>639</v>
-      </c>
-      <c r="E19" s="6"/>
+        <v>760</v>
+      </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="6" t="s">
-        <v>640</v>
+        <v>761</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>641</v>
+        <v>762</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>642</v>
-      </c>
-      <c r="E20" s="6"/>
+        <v>763</v>
+      </c>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="6" t="s">
-        <v>643</v>
+        <v>764</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>644</v>
+        <v>765</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>645</v>
-      </c>
-      <c r="E21" s="6"/>
+        <v>766</v>
+      </c>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="6" t="s">
-        <v>646</v>
+        <v>767</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>647</v>
+        <v>768</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>648</v>
-      </c>
-      <c r="E22" s="6"/>
+        <v>769</v>
+      </c>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="6" t="s">
-        <v>649</v>
+        <v>770</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>650</v>
+        <v>771</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>651</v>
-      </c>
-      <c r="E23" s="6"/>
+        <v>772</v>
+      </c>
     </row>
     <row r="24" spans="2:5">
       <c r="B24" s="6" t="s">
-        <v>652</v>
+        <v>773</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>653</v>
+        <v>774</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>654</v>
-      </c>
-      <c r="E24" s="6"/>
+        <v>775</v>
+      </c>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="6" t="s">
-        <v>655</v>
+        <v>776</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>656</v>
+        <v>777</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>657</v>
-      </c>
-      <c r="E25" s="6"/>
+        <v>778</v>
+      </c>
     </row>
     <row r="26" spans="2:5">
       <c r="B26" s="6" t="s">
-        <v>658</v>
+        <v>779</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>659</v>
+        <v>780</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="E26" s="6"/>
+        <v>781</v>
+      </c>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="6" t="s">
-        <v>661</v>
+        <v>782</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>662</v>
+        <v>783</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>663</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>664</v>
+        <v>784</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>785</v>
       </c>
     </row>
     <row r="28" spans="2:5">
       <c r="B28" s="6" t="s">
-        <v>665</v>
+        <v>786</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>666</v>
+        <v>787</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>667</v>
-      </c>
-      <c r="E28" s="6"/>
+        <v>788</v>
+      </c>
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="6" t="s">
-        <v>668</v>
+        <v>789</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>669</v>
+        <v>790</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>670</v>
-      </c>
-      <c r="E29" s="6"/>
+        <v>791</v>
+      </c>
     </row>
     <row r="30" spans="2:5">
       <c r="B30" s="6" t="s">
-        <v>671</v>
+        <v>792</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>672</v>
+        <v>793</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>673</v>
-      </c>
-      <c r="E30" s="6"/>
+        <v>794</v>
+      </c>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="6" t="s">
-        <v>674</v>
+        <v>795</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>675</v>
+        <v>796</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>676</v>
-      </c>
-      <c r="E31" s="6"/>
+        <v>797</v>
+      </c>
     </row>
     <row r="32" spans="2:5">
       <c r="B32" s="6" t="s">
-        <v>677</v>
+        <v>798</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>678</v>
+        <v>799</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>679</v>
-      </c>
-      <c r="E32" s="6"/>
+        <v>800</v>
+      </c>
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="6" t="s">
-        <v>680</v>
+        <v>801</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>681</v>
+        <v>802</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>682</v>
-      </c>
-      <c r="E33" s="6"/>
+        <v>803</v>
+      </c>
     </row>
     <row r="34" spans="2:5">
       <c r="B34" s="6" t="s">
-        <v>683</v>
+        <v>804</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>684</v>
+        <v>805</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>685</v>
-      </c>
-      <c r="E34" s="6"/>
+        <v>806</v>
+      </c>
     </row>
     <row r="35" spans="2:5">
       <c r="B35" s="6" t="s">
-        <v>686</v>
+        <v>807</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>687</v>
+        <v>808</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>688</v>
-      </c>
-      <c r="E35" s="6"/>
+        <v>809</v>
+      </c>
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="6" t="s">
-        <v>689</v>
+        <v>810</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>690</v>
+        <v>811</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>691</v>
-      </c>
-      <c r="E36" s="6"/>
+        <v>812</v>
+      </c>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="6" t="s">
-        <v>692</v>
+        <v>813</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>693</v>
+        <v>814</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>694</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>695</v>
+        <v>815</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>816</v>
       </c>
     </row>
     <row r="38" spans="2:5">
       <c r="B38" s="6" t="s">
-        <v>696</v>
+        <v>817</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>697</v>
+        <v>818</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>698</v>
-      </c>
-      <c r="E38" s="6"/>
+        <v>819</v>
+      </c>
     </row>
     <row r="39" spans="2:5">
       <c r="B39" s="6" t="s">
-        <v>699</v>
+        <v>820</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>700</v>
+        <v>821</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>701</v>
-      </c>
-      <c r="E39" s="6"/>
+        <v>822</v>
+      </c>
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="6" t="s">
-        <v>702</v>
+        <v>823</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>703</v>
+        <v>824</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>704</v>
-      </c>
-      <c r="E40" s="6"/>
+        <v>825</v>
+      </c>
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="6" t="s">
-        <v>705</v>
+        <v>826</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>706</v>
+        <v>827</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>707</v>
-      </c>
-      <c r="E41" s="6"/>
+        <v>828</v>
+      </c>
     </row>
     <row r="42" spans="2:5">
       <c r="B42" s="6" t="s">
-        <v>708</v>
+        <v>829</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>709</v>
+        <v>830</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>710</v>
-      </c>
-      <c r="E42" s="6"/>
+        <v>831</v>
+      </c>
     </row>
     <row r="43" spans="2:5">
       <c r="B43" s="6" t="s">
-        <v>711</v>
+        <v>832</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>712</v>
+        <v>833</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>713</v>
-      </c>
-      <c r="E43" s="6"/>
+        <v>834</v>
+      </c>
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="6" t="s">
-        <v>714</v>
+        <v>835</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>715</v>
+        <v>836</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>716</v>
-      </c>
-      <c r="E44" s="6"/>
+        <v>837</v>
+      </c>
     </row>
     <row r="45" spans="2:5">
       <c r="B45" s="6" t="s">
-        <v>717</v>
+        <v>838</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>718</v>
+        <v>839</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>719</v>
-      </c>
-      <c r="E45" s="6"/>
+        <v>840</v>
+      </c>
     </row>
     <row r="46" spans="2:5">
       <c r="B46" s="6" t="s">
-        <v>720</v>
+        <v>841</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>721</v>
+        <v>842</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>722</v>
-      </c>
-      <c r="E46" s="6"/>
+        <v>843</v>
+      </c>
     </row>
     <row r="47" spans="2:5">
       <c r="B47" s="6" t="s">
-        <v>723</v>
+        <v>844</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>724</v>
+        <v>845</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>725</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>726</v>
+        <v>846</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>847</v>
       </c>
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="6" t="s">
-        <v>727</v>
+        <v>848</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>728</v>
+        <v>849</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="E48" s="6"/>
+        <v>850</v>
+      </c>
     </row>
     <row r="49" spans="2:5">
       <c r="B49" s="6" t="s">
-        <v>730</v>
+        <v>851</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>731</v>
+        <v>852</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>732</v>
-      </c>
-      <c r="E49" s="6"/>
+        <v>853</v>
+      </c>
     </row>
     <row r="50" spans="2:5">
       <c r="B50" s="6" t="s">
-        <v>733</v>
+        <v>854</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>734</v>
+        <v>855</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>735</v>
-      </c>
-      <c r="E50" s="6"/>
+        <v>856</v>
+      </c>
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="6" t="s">
-        <v>736</v>
+        <v>857</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>737</v>
+        <v>858</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>738</v>
-      </c>
-      <c r="E51" s="6"/>
+        <v>859</v>
+      </c>
     </row>
     <row r="52" spans="2:5">
       <c r="B52" s="6" t="s">
-        <v>739</v>
+        <v>860</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>740</v>
+        <v>861</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>741</v>
-      </c>
-      <c r="E52" s="6"/>
+        <v>862</v>
+      </c>
     </row>
     <row r="53" spans="2:5">
       <c r="B53" s="6" t="s">
-        <v>742</v>
+        <v>863</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>743</v>
+        <v>864</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>744</v>
-      </c>
-      <c r="E53" s="6"/>
+        <v>865</v>
+      </c>
     </row>
     <row r="54" spans="2:5">
       <c r="B54" s="6" t="s">
-        <v>745</v>
+        <v>866</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>746</v>
+        <v>867</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>747</v>
-      </c>
-      <c r="E54" s="6"/>
+        <v>868</v>
+      </c>
     </row>
     <row r="55" spans="2:5">
       <c r="B55" s="6" t="s">
-        <v>748</v>
+        <v>869</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>749</v>
+        <v>870</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>750</v>
-      </c>
-      <c r="E55" s="6"/>
+        <v>871</v>
+      </c>
     </row>
     <row r="56" spans="2:5">
       <c r="B56" s="6" t="s">
-        <v>751</v>
+        <v>872</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>752</v>
+        <v>873</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>753</v>
-      </c>
-      <c r="E56" s="6"/>
+        <v>874</v>
+      </c>
     </row>
     <row r="57" spans="2:5">
       <c r="B57" s="6" t="s">
-        <v>754</v>
+        <v>875</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>755</v>
+        <v>876</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>756</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>757</v>
+        <v>877</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>878</v>
       </c>
     </row>
     <row r="58" spans="2:5">
       <c r="B58" s="6" t="s">
-        <v>758</v>
+        <v>879</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>759</v>
+        <v>880</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>760</v>
-      </c>
-      <c r="E58" s="6"/>
+        <v>881</v>
+      </c>
     </row>
     <row r="59" spans="2:5">
       <c r="B59" s="6" t="s">
-        <v>761</v>
+        <v>882</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>762</v>
+        <v>883</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>763</v>
-      </c>
-      <c r="E59" s="6"/>
+        <v>884</v>
+      </c>
     </row>
     <row r="60" spans="2:5">
       <c r="B60" s="6" t="s">
-        <v>764</v>
+        <v>885</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>765</v>
+        <v>886</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>766</v>
-      </c>
-      <c r="E60" s="6"/>
+        <v>887</v>
+      </c>
     </row>
     <row r="61" spans="2:5">
       <c r="B61" s="6" t="s">
-        <v>767</v>
+        <v>888</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>768</v>
+        <v>889</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>769</v>
-      </c>
-      <c r="E61" s="6"/>
+        <v>890</v>
+      </c>
     </row>
     <row r="62" spans="2:5">
       <c r="B62" s="6" t="s">
-        <v>770</v>
+        <v>891</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>771</v>
+        <v>892</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>772</v>
-      </c>
-      <c r="E62" s="6"/>
+        <v>893</v>
+      </c>
     </row>
     <row r="63" spans="2:5">
       <c r="B63" s="6" t="s">
-        <v>773</v>
+        <v>894</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>774</v>
+        <v>895</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>775</v>
-      </c>
-      <c r="E63" s="6"/>
+        <v>896</v>
+      </c>
     </row>
     <row r="64" spans="2:5">
       <c r="B64" s="6" t="s">
-        <v>776</v>
+        <v>897</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>777</v>
+        <v>898</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>778</v>
-      </c>
-      <c r="E64" s="6"/>
+        <v>899</v>
+      </c>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="6" t="s">
-        <v>779</v>
+        <v>900</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>780</v>
+        <v>901</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>781</v>
-      </c>
-      <c r="E65" s="6"/>
+        <v>902</v>
+      </c>
     </row>
     <row r="66" spans="2:5">
       <c r="B66" s="6" t="s">
-        <v>782</v>
+        <v>903</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>783</v>
+        <v>904</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>784</v>
-      </c>
-      <c r="E66" s="6"/>
+        <v>905</v>
+      </c>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="6" t="s">
-        <v>785</v>
+        <v>906</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>786</v>
+        <v>907</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>787</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>788</v>
+        <v>908</v>
+      </c>
+      <c r="E67" s="12" t="s">
+        <v>909</v>
       </c>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="6" t="s">
-        <v>789</v>
+        <v>910</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>790</v>
+        <v>911</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>791</v>
-      </c>
-      <c r="E68" s="6"/>
+        <v>912</v>
+      </c>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="6" t="s">
-        <v>792</v>
+        <v>913</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>793</v>
+        <v>914</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>794</v>
-      </c>
-      <c r="E69" s="6"/>
+        <v>915</v>
+      </c>
     </row>
     <row r="70" spans="2:5">
       <c r="B70" s="6" t="s">
-        <v>795</v>
+        <v>916</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>796</v>
+        <v>917</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>797</v>
-      </c>
-      <c r="E70" s="6"/>
+        <v>918</v>
+      </c>
     </row>
     <row r="71" spans="2:5">
       <c r="B71" s="6" t="s">
-        <v>798</v>
+        <v>919</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>799</v>
+        <v>920</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>800</v>
-      </c>
-      <c r="E71" s="6"/>
+        <v>921</v>
+      </c>
     </row>
     <row r="72" spans="2:5">
       <c r="B72" s="6" t="s">
-        <v>801</v>
+        <v>922</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>802</v>
+        <v>923</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>803</v>
-      </c>
-      <c r="E72" s="6"/>
+        <v>924</v>
+      </c>
     </row>
     <row r="73" spans="2:5">
       <c r="B73" s="6" t="s">
-        <v>804</v>
+        <v>925</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>805</v>
+        <v>926</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>806</v>
-      </c>
-      <c r="E73" s="6"/>
+        <v>927</v>
+      </c>
     </row>
     <row r="74" spans="2:5">
       <c r="B74" s="6" t="s">
-        <v>807</v>
+        <v>928</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>808</v>
+        <v>929</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>809</v>
-      </c>
-      <c r="E74" s="6"/>
+        <v>930</v>
+      </c>
     </row>
     <row r="75" spans="2:5">
       <c r="B75" s="6" t="s">
-        <v>810</v>
+        <v>931</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>811</v>
+        <v>932</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>812</v>
-      </c>
-      <c r="E75" s="6"/>
+        <v>933</v>
+      </c>
     </row>
     <row r="76" spans="2:5">
       <c r="B76" s="6" t="s">
-        <v>813</v>
+        <v>934</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>814</v>
+        <v>935</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>815</v>
-      </c>
-      <c r="E76" s="6"/>
+        <v>936</v>
+      </c>
     </row>
     <row r="77" spans="2:5">
       <c r="B77" s="6" t="s">
-        <v>816</v>
+        <v>937</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>817</v>
+        <v>938</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>818</v>
-      </c>
-      <c r="E77" s="6" t="s">
-        <v>819</v>
+        <v>939</v>
+      </c>
+      <c r="E77" s="12" t="s">
+        <v>940</v>
       </c>
     </row>
     <row r="78" spans="2:5">
       <c r="B78" s="6" t="s">
-        <v>820</v>
+        <v>941</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>821</v>
+        <v>942</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>822</v>
-      </c>
-      <c r="E78" s="6"/>
+        <v>943</v>
+      </c>
     </row>
     <row r="79" spans="2:5">
       <c r="B79" s="6" t="s">
-        <v>823</v>
+        <v>944</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>824</v>
+        <v>945</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>825</v>
-      </c>
-      <c r="E79" s="6"/>
+        <v>946</v>
+      </c>
     </row>
     <row r="80" spans="2:5">
       <c r="B80" s="6" t="s">
-        <v>826</v>
+        <v>947</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>827</v>
+        <v>948</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>828</v>
-      </c>
-      <c r="E80" s="6"/>
+        <v>949</v>
+      </c>
     </row>
     <row r="81" spans="2:5">
       <c r="B81" s="6" t="s">
-        <v>829</v>
+        <v>950</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>830</v>
+        <v>951</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>831</v>
-      </c>
-      <c r="E81" s="6"/>
+        <v>952</v>
+      </c>
     </row>
     <row r="82" spans="2:5">
       <c r="B82" s="6" t="s">
-        <v>832</v>
+        <v>953</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>833</v>
+        <v>954</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>834</v>
-      </c>
-      <c r="E82" s="6"/>
+        <v>955</v>
+      </c>
     </row>
     <row r="83" spans="2:5">
       <c r="B83" s="6" t="s">
-        <v>835</v>
+        <v>956</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>836</v>
+        <v>957</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>837</v>
-      </c>
-      <c r="E83" s="6"/>
+        <v>958</v>
+      </c>
     </row>
     <row r="84" spans="2:5">
       <c r="B84" s="6" t="s">
-        <v>838</v>
+        <v>959</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>839</v>
+        <v>960</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>840</v>
-      </c>
-      <c r="E84" s="6"/>
+        <v>961</v>
+      </c>
     </row>
     <row r="85" spans="2:5">
       <c r="B85" s="6" t="s">
-        <v>841</v>
+        <v>962</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>842</v>
+        <v>963</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>843</v>
-      </c>
-      <c r="E85" s="6"/>
+        <v>964</v>
+      </c>
     </row>
     <row r="86" spans="2:5">
       <c r="B86" s="6" t="s">
-        <v>844</v>
+        <v>965</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>845</v>
+        <v>966</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>846</v>
-      </c>
-      <c r="E86" s="6"/>
+        <v>967</v>
+      </c>
     </row>
     <row r="87" spans="2:5">
       <c r="B87" s="6" t="s">
-        <v>847</v>
+        <v>968</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>848</v>
+        <v>969</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>849</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>850</v>
+        <v>970</v>
+      </c>
+      <c r="E87" s="12" t="s">
+        <v>971</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J107"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" style="6" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" style="6" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>851</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>852</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>853</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="24" customHeight="1">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>852</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>854</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>852</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>854</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>856</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>857</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>858</v>
-      </c>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7" spans="1:10" ht="42" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="B8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>425</v>
-      </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="B9" s="6" t="s">
-        <v>859</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>860</v>
-      </c>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="B10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>861</v>
-      </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="B11" s="6" t="s">
-        <v>433</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>862</v>
-      </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="B12" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>863</v>
-      </c>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="B13" s="6" t="s">
-        <v>443</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>864</v>
-      </c>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="B14" s="6" t="s">
-        <v>865</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>866</v>
-      </c>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="B15" s="6" t="s">
-        <v>867</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>868</v>
-      </c>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="B16" s="6" t="s">
-        <v>456</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>869</v>
-      </c>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="2:4">
-      <c r="B17" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>870</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4">
-      <c r="B18" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>872</v>
-      </c>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" spans="2:4">
-      <c r="B19" s="6" t="s">
-        <v>873</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>874</v>
-      </c>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20" spans="2:4">
-      <c r="B20" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>875</v>
-      </c>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21" spans="2:4">
-      <c r="B21" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>876</v>
-      </c>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22" spans="2:4">
-      <c r="B22" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>877</v>
-      </c>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23" spans="2:4">
-      <c r="B23" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>878</v>
-      </c>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" spans="2:4">
-      <c r="B24" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>879</v>
-      </c>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="2:4">
-      <c r="B25" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>880</v>
-      </c>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26" spans="2:4">
-      <c r="B26" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>881</v>
-      </c>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27" spans="2:4">
-      <c r="B27" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>882</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>883</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4">
-      <c r="B28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>884</v>
-      </c>
-      <c r="D28" s="6"/>
-    </row>
-    <row r="29" spans="2:4">
-      <c r="B29" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>885</v>
-      </c>
-      <c r="D29" s="6"/>
-    </row>
-    <row r="30" spans="2:4">
-      <c r="B30" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>886</v>
-      </c>
-      <c r="D30" s="6"/>
-    </row>
-    <row r="31" spans="2:4">
-      <c r="B31" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>887</v>
-      </c>
-      <c r="D31" s="6"/>
-    </row>
-    <row r="32" spans="2:4">
-      <c r="B32" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>888</v>
-      </c>
-      <c r="D32" s="6"/>
-    </row>
-    <row r="33" spans="2:4">
-      <c r="B33" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>889</v>
-      </c>
-      <c r="D33" s="6"/>
-    </row>
-    <row r="34" spans="2:4">
-      <c r="B34" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>890</v>
-      </c>
-      <c r="D34" s="6"/>
-    </row>
-    <row r="35" spans="2:4">
-      <c r="B35" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>891</v>
-      </c>
-      <c r="D35" s="6"/>
-    </row>
-    <row r="36" spans="2:4">
-      <c r="B36" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>892</v>
-      </c>
-      <c r="D36" s="6"/>
-    </row>
-    <row r="37" spans="2:4">
-      <c r="B37" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>893</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>894</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4">
-      <c r="B38" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>895</v>
-      </c>
-      <c r="D38" s="6"/>
-    </row>
-    <row r="39" spans="2:4">
-      <c r="B39" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>896</v>
-      </c>
-      <c r="D39" s="6"/>
-    </row>
-    <row r="40" spans="2:4">
-      <c r="B40" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>897</v>
-      </c>
-      <c r="D40" s="6"/>
-    </row>
-    <row r="41" spans="2:4">
-      <c r="B41" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>898</v>
-      </c>
-      <c r="D41" s="6"/>
-    </row>
-    <row r="42" spans="2:4">
-      <c r="B42" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>899</v>
-      </c>
-      <c r="D42" s="6"/>
-    </row>
-    <row r="43" spans="2:4">
-      <c r="B43" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>900</v>
-      </c>
-      <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="2:4">
-      <c r="B44" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>901</v>
-      </c>
-      <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="2:4">
-      <c r="B45" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>902</v>
-      </c>
-      <c r="D45" s="6"/>
-    </row>
-    <row r="46" spans="2:4">
-      <c r="B46" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>903</v>
-      </c>
-      <c r="D46" s="6"/>
-    </row>
-    <row r="47" spans="2:4">
-      <c r="B47" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>904</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="48" spans="2:4">
-      <c r="B48" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>906</v>
-      </c>
-      <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="2:4">
-      <c r="B49" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>907</v>
-      </c>
-      <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="2:4">
-      <c r="B50" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>908</v>
-      </c>
-      <c r="D50" s="6"/>
-    </row>
-    <row r="51" spans="2:4">
-      <c r="B51" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>909</v>
-      </c>
-      <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="2:4">
-      <c r="B52" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>910</v>
-      </c>
-      <c r="D52" s="6"/>
-    </row>
-    <row r="53" spans="2:4">
-      <c r="B53" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>911</v>
-      </c>
-      <c r="D53" s="6"/>
-    </row>
-    <row r="54" spans="2:4">
-      <c r="B54" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>912</v>
-      </c>
-      <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="2:4">
-      <c r="B55" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>913</v>
-      </c>
-      <c r="D55" s="6"/>
-    </row>
-    <row r="56" spans="2:4">
-      <c r="B56" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>914</v>
-      </c>
-      <c r="D56" s="6"/>
-    </row>
-    <row r="57" spans="2:4">
-      <c r="B57" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>915</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>916</v>
-      </c>
-    </row>
-    <row r="58" spans="2:4">
-      <c r="B58" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>917</v>
-      </c>
-      <c r="D58" s="6"/>
-    </row>
-    <row r="59" spans="2:4">
-      <c r="B59" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>918</v>
-      </c>
-      <c r="D59" s="6"/>
-    </row>
-    <row r="60" spans="2:4">
-      <c r="B60" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>919</v>
-      </c>
-      <c r="D60" s="6"/>
-    </row>
-    <row r="61" spans="2:4">
-      <c r="B61" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>920</v>
-      </c>
-      <c r="D61" s="6"/>
-    </row>
-    <row r="62" spans="2:4">
-      <c r="B62" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>921</v>
-      </c>
-      <c r="D62" s="6"/>
-    </row>
-    <row r="63" spans="2:4">
-      <c r="B63" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>922</v>
-      </c>
-      <c r="D63" s="6"/>
-    </row>
-    <row r="64" spans="2:4">
-      <c r="B64" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>923</v>
-      </c>
-      <c r="D64" s="6"/>
-    </row>
-    <row r="65" spans="2:4">
-      <c r="B65" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>924</v>
-      </c>
-      <c r="D65" s="6"/>
-    </row>
-    <row r="66" spans="2:4">
-      <c r="B66" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>925</v>
-      </c>
-      <c r="D66" s="6"/>
-    </row>
-    <row r="67" spans="2:4">
-      <c r="B67" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>926</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>927</v>
-      </c>
-    </row>
-    <row r="68" spans="2:4">
-      <c r="B68" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>928</v>
-      </c>
-      <c r="D68" s="6"/>
-    </row>
-    <row r="69" spans="2:4">
-      <c r="B69" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>929</v>
-      </c>
-      <c r="D69" s="6"/>
-    </row>
-    <row r="70" spans="2:4">
-      <c r="B70" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>930</v>
-      </c>
-      <c r="D70" s="6"/>
-    </row>
-    <row r="71" spans="2:4">
-      <c r="B71" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>931</v>
-      </c>
-      <c r="D71" s="6"/>
-    </row>
-    <row r="72" spans="2:4">
-      <c r="B72" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>932</v>
-      </c>
-      <c r="D72" s="6"/>
-    </row>
-    <row r="73" spans="2:4">
-      <c r="B73" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>933</v>
-      </c>
-      <c r="D73" s="6"/>
-    </row>
-    <row r="74" spans="2:4">
-      <c r="B74" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>934</v>
-      </c>
-      <c r="D74" s="6"/>
-    </row>
-    <row r="75" spans="2:4">
-      <c r="B75" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>935</v>
-      </c>
-      <c r="D75" s="6"/>
-    </row>
-    <row r="76" spans="2:4">
-      <c r="B76" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>936</v>
-      </c>
-      <c r="D76" s="6"/>
-    </row>
-    <row r="77" spans="2:4">
-      <c r="B77" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>937</v>
-      </c>
-      <c r="D77" s="6" t="s">
-        <v>938</v>
-      </c>
-    </row>
-    <row r="78" spans="2:4">
-      <c r="B78" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>939</v>
-      </c>
-      <c r="D78" s="6"/>
-    </row>
-    <row r="79" spans="2:4">
-      <c r="B79" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>940</v>
-      </c>
-      <c r="D79" s="6"/>
-    </row>
-    <row r="80" spans="2:4">
-      <c r="B80" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="C80" s="6" t="s">
-        <v>941</v>
-      </c>
-      <c r="D80" s="6"/>
-    </row>
-    <row r="81" spans="2:4">
-      <c r="B81" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>942</v>
-      </c>
-      <c r="D81" s="6"/>
-    </row>
-    <row r="82" spans="2:4">
-      <c r="B82" s="6" t="s">
-        <v>322</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>943</v>
-      </c>
-      <c r="D82" s="6"/>
-    </row>
-    <row r="83" spans="2:4">
-      <c r="B83" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>944</v>
-      </c>
-      <c r="D83" s="6"/>
-    </row>
-    <row r="84" spans="2:4">
-      <c r="B84" s="6" t="s">
-        <v>334</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>945</v>
-      </c>
-      <c r="D84" s="6"/>
-    </row>
-    <row r="85" spans="2:4">
-      <c r="B85" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>946</v>
-      </c>
-      <c r="D85" s="6"/>
-    </row>
-    <row r="86" spans="2:4">
-      <c r="B86" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>947</v>
-      </c>
-      <c r="D86" s="6"/>
-    </row>
-    <row r="87" spans="2:4">
-      <c r="B87" s="6" t="s">
-        <v>342</v>
-      </c>
-      <c r="C87" s="6" t="s">
-        <v>948</v>
-      </c>
-      <c r="D87" s="6" t="s">
-        <v>949</v>
-      </c>
-    </row>
-    <row r="88" spans="2:4">
-      <c r="B88" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>950</v>
-      </c>
-      <c r="D88" s="6"/>
-    </row>
-    <row r="89" spans="2:4">
-      <c r="B89" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="C89" s="6" t="s">
-        <v>951</v>
-      </c>
-      <c r="D89" s="6"/>
-    </row>
-    <row r="90" spans="2:4">
-      <c r="B90" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="C90" s="6" t="s">
-        <v>952</v>
-      </c>
-      <c r="D90" s="6"/>
-    </row>
-    <row r="91" spans="2:4">
-      <c r="B91" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>953</v>
-      </c>
-      <c r="D91" s="6"/>
-    </row>
-    <row r="92" spans="2:4">
-      <c r="B92" s="6" t="s">
-        <v>362</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>954</v>
-      </c>
-      <c r="D92" s="6"/>
-    </row>
-    <row r="93" spans="2:4">
-      <c r="B93" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>955</v>
-      </c>
-      <c r="D93" s="6"/>
-    </row>
-    <row r="94" spans="2:4">
-      <c r="B94" s="6" t="s">
-        <v>374</v>
-      </c>
-      <c r="C94" s="6" t="s">
-        <v>956</v>
-      </c>
-      <c r="D94" s="6"/>
-    </row>
-    <row r="95" spans="2:4">
-      <c r="B95" s="6" t="s">
-        <v>373</v>
-      </c>
-      <c r="C95" s="6" t="s">
-        <v>957</v>
-      </c>
-      <c r="D95" s="6"/>
-    </row>
-    <row r="96" spans="2:4">
-      <c r="B96" s="6" t="s">
-        <v>378</v>
-      </c>
-      <c r="C96" s="6" t="s">
-        <v>958</v>
-      </c>
-      <c r="D96" s="6"/>
-    </row>
-    <row r="97" spans="2:4">
-      <c r="B97" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="C97" s="6" t="s">
-        <v>959</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>960</v>
-      </c>
-    </row>
-    <row r="98" spans="2:4">
-      <c r="B98" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C98" s="6" t="s">
-        <v>961</v>
-      </c>
-      <c r="D98" s="6"/>
-    </row>
-    <row r="99" spans="2:4">
-      <c r="B99" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="C99" s="6" t="s">
-        <v>962</v>
-      </c>
-      <c r="D99" s="6"/>
-    </row>
-    <row r="100" spans="2:4">
-      <c r="B100" s="6" t="s">
-        <v>393</v>
-      </c>
-      <c r="C100" s="6" t="s">
-        <v>963</v>
-      </c>
-      <c r="D100" s="6"/>
-    </row>
-    <row r="101" spans="2:4">
-      <c r="B101" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="C101" s="6" t="s">
-        <v>964</v>
-      </c>
-      <c r="D101" s="6"/>
-    </row>
-    <row r="102" spans="2:4">
-      <c r="B102" s="6" t="s">
-        <v>402</v>
-      </c>
-      <c r="C102" s="6" t="s">
-        <v>965</v>
-      </c>
-      <c r="D102" s="6"/>
-    </row>
-    <row r="103" spans="2:4">
-      <c r="B103" s="6" t="s">
-        <v>409</v>
-      </c>
-      <c r="C103" s="6" t="s">
-        <v>966</v>
-      </c>
-      <c r="D103" s="6"/>
-    </row>
-    <row r="104" spans="2:4">
-      <c r="B104" s="6" t="s">
-        <v>414</v>
-      </c>
-      <c r="C104" s="6" t="s">
-        <v>967</v>
-      </c>
-      <c r="D104" s="6"/>
-    </row>
-    <row r="105" spans="2:4">
-      <c r="B105" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="C105" s="6" t="s">
-        <v>968</v>
-      </c>
-      <c r="D105" s="6"/>
-    </row>
-    <row r="106" spans="2:4">
-      <c r="B106" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="C106" s="6" t="s">
-        <v>969</v>
-      </c>
-      <c r="D106" s="6"/>
-    </row>
-    <row r="107" spans="2:4">
-      <c r="B107" s="6" t="s">
-        <v>425</v>
-      </c>
-      <c r="C107" s="6" t="s">
-        <v>970</v>
-      </c>
-      <c r="D107" s="6" t="s">
-        <v>971</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 100." promptTitle="Integer range" prompt="Enter an integer from 1 to 100." sqref="B8:B1007">
-      <formula1>1</formula1>
-      <formula2>100</formula2>
-    </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 999999999." promptTitle="Integer range" prompt="Enter an integer from 0 to 999999999." sqref="C8:C1007">
-      <formula1>0</formula1>
-      <formula2>999999999</formula2>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>